<commit_message>
code updated for vehicle paper plan
https://docs.google.com/presentation/d/1vR-Z3FztOdoZGlURnNq2B7ZdfjmG5KwprPIkB8TYwGc/edit?usp=sharing
</commit_message>
<xml_diff>
--- a/code/output/vehicle_model_results.xlsx
+++ b/code/output/vehicle_model_results.xlsx
@@ -1,24 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Spring 2025\Conjoint_Survey_25\code\output\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7089E4E-6D08-4747-B34E-DC8AA72C16F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1506456D-8A0C-4EF5-BF55-36C862BCE8CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="4" xr2:uid="{7CCC4083-8FE9-4953-9603-647056C47B46}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="3" xr2:uid="{7CCC4083-8FE9-4953-9603-647056C47B46}"/>
   </bookViews>
   <sheets>
     <sheet name="model car || suv" sheetId="4" r:id="rId1"/>
     <sheet name="wtp models-low || high" sheetId="1" r:id="rId2"/>
     <sheet name="conf intervals-low || high" sheetId="2" r:id="rId3"/>
-    <sheet name="models-interaction" sheetId="3" r:id="rId4"/>
-    <sheet name="conf intervals - interaction" sheetId="6" r:id="rId5"/>
-    <sheet name="models_log_r" sheetId="5" r:id="rId6"/>
+    <sheet name="models pro_averse" sheetId="7" r:id="rId4"/>
+    <sheet name="models-interaction" sheetId="3" r:id="rId5"/>
+    <sheet name="conf intervals - interaction" sheetId="6" r:id="rId6"/>
+    <sheet name="models_log_r" sheetId="5" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="502" uniqueCount="382">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="572" uniqueCount="378">
   <si>
     <t xml:space="preserve">Model Coefficients: </t>
   </si>
@@ -85,228 +86,33 @@
     <t xml:space="preserve">                 Estimate Std. Error  z-value  Pr(&gt;|z|)    </t>
   </si>
   <si>
-    <t>scalePar        2.0544116  0.1039379  19.7658 &lt; 2.2e-16 ***</t>
-  </si>
-  <si>
-    <t>no_choice      -3.2091109  0.1256547 -25.5391 &lt; 2.2e-16 ***</t>
-  </si>
-  <si>
-    <t>powertrainbev  -0.8300578  0.1000585  -8.2957 &lt; 2.2e-16 ***</t>
-  </si>
-  <si>
-    <t>powertrainhev  -0.1824343  0.0426388  -4.2786 1.881e-05 ***</t>
-  </si>
-  <si>
-    <t xml:space="preserve">range_bev       0.0439657  0.0767928   0.5725  0.566967    </t>
-  </si>
-  <si>
-    <t>mileage        -0.1058290  0.0128262  -8.2510 2.220e-16 ***</t>
-  </si>
-  <si>
-    <t>age            -0.0237303  0.0070256  -3.3777  0.000731 ***</t>
-  </si>
-  <si>
-    <t>operating_cost -0.4186492  0.0538337  -7.7767 7.550e-15 ***</t>
-  </si>
-  <si>
-    <t>Log-Likelihood:         -2132.3693139</t>
-  </si>
-  <si>
     <t>Null Log-Likelihood:    -2661.6851734</t>
   </si>
   <si>
-    <t>AIC:                     4280.7386279</t>
-  </si>
-  <si>
-    <t>BIC:                     4325.2193000</t>
-  </si>
-  <si>
-    <t>McFadden R2:                0.1988649</t>
-  </si>
-  <si>
-    <t>Adj McFadden R2:            0.1958593</t>
-  </si>
-  <si>
     <t>Number of Observations:  1920.0000000</t>
   </si>
   <si>
-    <t>scalePar        0.857060   0.061742  13.8813 &lt; 2.2e-16 ***</t>
-  </si>
-  <si>
-    <t>no_choice      -6.395621   0.369940 -17.2883 &lt; 2.2e-16 ***</t>
-  </si>
-  <si>
-    <t>powertrainbev  -2.151756   0.378985  -5.6777 1.365e-08 ***</t>
-  </si>
-  <si>
-    <t xml:space="preserve">powertrainhev   0.125884   0.129428   0.9726    0.3307    </t>
-  </si>
-  <si>
-    <t>range_bev       0.709486   0.170049   4.1722 3.016e-05 ***</t>
-  </si>
-  <si>
-    <t>mileage        -0.279548   0.040789  -6.8535 7.206e-12 ***</t>
-  </si>
-  <si>
-    <t>age            -0.154868   0.022988  -6.7370 1.617e-11 ***</t>
-  </si>
-  <si>
-    <t>operating_cost -0.769709   0.167366  -4.5990 4.246e-06 ***</t>
-  </si>
-  <si>
-    <t>Log-Likelihood:         -1363.3994577</t>
-  </si>
-  <si>
     <t>Null Log-Likelihood:    -1597.0111040</t>
   </si>
   <si>
-    <t>AIC:                     2742.7989155</t>
-  </si>
-  <si>
-    <t>BIC:                     2783.1930000</t>
-  </si>
-  <si>
-    <t>McFadden R2:                0.1462805</t>
-  </si>
-  <si>
-    <t>Adj McFadden R2:            0.1412712</t>
-  </si>
-  <si>
     <t>Number of Observations:  1152.0000000</t>
   </si>
   <si>
-    <t>scalePar        1.423647   0.098213  14.4954 &lt; 2.2e-16 ***</t>
-  </si>
-  <si>
-    <t>no_choice      -4.235841   0.213589 -19.8318 &lt; 2.2e-16 ***</t>
-  </si>
-  <si>
-    <t>powertrainbev  -1.990338   0.313966  -6.3393 2.307e-10 ***</t>
-  </si>
-  <si>
-    <t xml:space="preserve">powertrainhev  -0.124603   0.060572  -2.0571 0.0396764 *  </t>
-  </si>
-  <si>
-    <t xml:space="preserve">range_bev       0.412597   0.136839   3.0152 0.0025681 ** </t>
-  </si>
-  <si>
-    <t>mileage        -0.152053   0.022958  -6.6231 3.516e-11 ***</t>
-  </si>
-  <si>
-    <t>age            -0.044340   0.012158  -3.6468 0.0002655 ***</t>
-  </si>
-  <si>
-    <t>operating_cost -0.536495   0.085368  -6.2845 3.289e-10 ***</t>
-  </si>
-  <si>
-    <t>Log-Likelihood:         -1582.4762171</t>
-  </si>
-  <si>
     <t>Null Log-Likelihood:    -1871.4973875</t>
   </si>
   <si>
-    <t>AIC:                     3180.9524343</t>
-  </si>
-  <si>
-    <t>BIC:                     3222.6153000</t>
-  </si>
-  <si>
-    <t>McFadden R2:                0.1544331</t>
-  </si>
-  <si>
-    <t>Adj McFadden R2:            0.1501585</t>
-  </si>
-  <si>
     <t>Number of Observations:  1350.0000000</t>
   </si>
   <si>
-    <t>scalePar        0.735680   0.045040  16.3339 &lt; 2.2e-16 ***</t>
-  </si>
-  <si>
-    <t>no_choice      -7.575005   0.342728 -22.1021 &lt; 2.2e-16 ***</t>
-  </si>
-  <si>
-    <t>powertrainbev  -2.658033   0.419451  -6.3369 2.344e-10 ***</t>
-  </si>
-  <si>
-    <t xml:space="preserve">powertrainhev   0.150874   0.099854   1.5109    0.1308    </t>
-  </si>
-  <si>
-    <t>range_bev       0.585427   0.133409   4.3882 1.143e-05 ***</t>
-  </si>
-  <si>
-    <t>mileage        -0.384054   0.038580  -9.9547 &lt; 2.2e-16 ***</t>
-  </si>
-  <si>
-    <t>age            -0.221201   0.021834 -10.1311 &lt; 2.2e-16 ***</t>
-  </si>
-  <si>
-    <t>operating_cost -0.722569   0.129566  -5.5769 2.449e-08 ***</t>
-  </si>
-  <si>
-    <t>Log-Likelihood:         -2589.0627849</t>
-  </si>
-  <si>
     <t>Null Log-Likelihood:    -2952.8069892</t>
   </si>
   <si>
-    <t>AIC:                     5194.1255698</t>
-  </si>
-  <si>
-    <t>BIC:                     5239.4366000</t>
-  </si>
-  <si>
-    <t>McFadden R2:                0.1231859</t>
-  </si>
-  <si>
-    <t>Adj McFadden R2:            0.1204766</t>
-  </si>
-  <si>
     <t>Number of Observations:  2130.0000000</t>
   </si>
   <si>
-    <t>powertrainbev  -1.943519   0.141915 -13.6949 &lt; 2.2e-16 ***</t>
-  </si>
-  <si>
-    <t xml:space="preserve">powertrainhev  -0.193907   0.066237  -2.9275  0.003417 ** </t>
-  </si>
-  <si>
-    <t>range_bev       0.553628   0.082058   6.7468 1.511e-11 ***</t>
-  </si>
-  <si>
-    <t>mileage        -0.213793   0.019286 -11.0852 &lt; 2.2e-16 ***</t>
-  </si>
-  <si>
-    <t>age            -0.077736   0.010972  -7.0848 1.392e-12 ***</t>
-  </si>
-  <si>
-    <t>operating_cost -0.735919   0.081843  -8.9919 &lt; 2.2e-16 ***</t>
-  </si>
-  <si>
-    <t>price          -0.963002   0.045134 -21.3363 &lt; 2.2e-16 ***</t>
-  </si>
-  <si>
-    <t>no_choice      -5.283851   0.193636 -27.2875 &lt; 2.2e-16 ***</t>
-  </si>
-  <si>
-    <t>Log-Likelihood:         -3601.4669820</t>
-  </si>
-  <si>
     <t>Null Log-Likelihood:    -4258.6962774</t>
   </si>
   <si>
-    <t>AIC:                     7218.9339641</t>
-  </si>
-  <si>
-    <t>BIC:                     7267.1746000</t>
-  </si>
-  <si>
-    <t>McFadden R2:                0.1543264</t>
-  </si>
-  <si>
-    <t>Adj McFadden R2:            0.1524479</t>
-  </si>
-  <si>
     <t>Number of Observations:  3072.0000000</t>
   </si>
   <si>
@@ -319,48 +125,9 @@
     <t xml:space="preserve">                 Estimate Std. Error  z-value Pr(&gt;|z|)    </t>
   </si>
   <si>
-    <t>powertrainbev  -2.5588692  0.1999209 -12.7994   &lt;2e-16 ***</t>
-  </si>
-  <si>
-    <t xml:space="preserve">powertrainhev  -0.0079799  0.0548839  -0.1454   0.8844    </t>
-  </si>
-  <si>
-    <t>range_bev       0.5979603  0.0713876   8.3763   &lt;2e-16 ***</t>
-  </si>
-  <si>
-    <t>mileage        -0.2537472  0.0186282 -13.6217   &lt;2e-16 ***</t>
-  </si>
-  <si>
-    <t>age            -0.1218759  0.0105121 -11.5938   &lt;2e-16 ***</t>
-  </si>
-  <si>
-    <t>operating_cost -0.6132787  0.0702199  -8.7337   &lt;2e-16 ***</t>
-  </si>
-  <si>
-    <t>price          -0.7175835  0.0360801 -19.8886   &lt;2e-16 ***</t>
-  </si>
-  <si>
-    <t>no_choice      -5.1985335  0.1864884 -27.8759   &lt;2e-16 ***</t>
-  </si>
-  <si>
-    <t>Log-Likelihood:         -4238.0927084</t>
-  </si>
-  <si>
     <t>Null Log-Likelihood:    -4824.3043767</t>
   </si>
   <si>
-    <t>AIC:                     8492.1854168</t>
-  </si>
-  <si>
-    <t>BIC:                     8541.4237000</t>
-  </si>
-  <si>
-    <t>McFadden R2:                0.1215122</t>
-  </si>
-  <si>
-    <t>Adj McFadden R2:            0.1198539</t>
-  </si>
-  <si>
     <t>Number of Observations:  3480.0000000</t>
   </si>
   <si>
@@ -892,129 +659,9 @@
     <t xml:space="preserve">                    mean     lower     upper</t>
   </si>
   <si>
-    <t>powertrainbev   -8315.31 -10337.71  -6411.11</t>
-  </si>
-  <si>
-    <t>powertrainhev   -1826.50  -2679.80  -1005.33</t>
-  </si>
-  <si>
-    <t>range_bev         432.57  -1065.40   1932.37</t>
-  </si>
-  <si>
-    <t>mileage         -1061.16  -1323.58   -812.89</t>
-  </si>
-  <si>
-    <t>age              -236.58   -376.21    -98.06</t>
-  </si>
-  <si>
-    <t>operating_cost  -4195.34  -5271.81  -3168.41</t>
-  </si>
-  <si>
     <t>price          -10000.00 -10000.00 -10000.00</t>
   </si>
   <si>
-    <t>no_choice      -32130.29 -34782.43 -29772.75</t>
-  </si>
-  <si>
-    <t>BEV100          -7882.74  -9127.79  -6713.86</t>
-  </si>
-  <si>
-    <t>BEV200          -7450.16  -9363.65  -5607.61</t>
-  </si>
-  <si>
-    <t>BEV300          -7017.59 -10254.84  -3872.13</t>
-  </si>
-  <si>
-    <t>powertrainbev  -21665.03 -29373.59 -14419.73</t>
-  </si>
-  <si>
-    <t>powertrainhev    1265.72  -1249.93   3802.49</t>
-  </si>
-  <si>
-    <t>range_bev        7150.58   3887.44  10577.71</t>
-  </si>
-  <si>
-    <t>mileage         -2805.16  -3664.14  -2038.10</t>
-  </si>
-  <si>
-    <t>age             -1553.31  -2027.93  -1125.87</t>
-  </si>
-  <si>
-    <t>operating_cost  -7726.30 -11229.67  -4504.82</t>
-  </si>
-  <si>
-    <t>no_choice      -64100.46 -71960.76 -57147.72</t>
-  </si>
-  <si>
-    <t>BEV100         -14514.44 -19324.94 -10048.56</t>
-  </si>
-  <si>
-    <t>BEV200          -7363.86 -10522.47  -4342.08</t>
-  </si>
-  <si>
-    <t>BEV300           -213.28  -4660.27   4328.72</t>
-  </si>
-  <si>
-    <t>powertrainbev  -26650.81 -35187.91 -18541.99</t>
-  </si>
-  <si>
-    <t>powertrainhev    1507.32   -473.80   3520.89</t>
-  </si>
-  <si>
-    <t>range_bev        5863.68   3234.84   8511.66</t>
-  </si>
-  <si>
-    <t>mileage         -3850.11  -4625.83  -3126.48</t>
-  </si>
-  <si>
-    <t>age             -2221.28  -2683.42  -1805.97</t>
-  </si>
-  <si>
-    <t>operating_cost  -7255.59  -9898.73  -4740.41</t>
-  </si>
-  <si>
-    <t>no_choice      -75909.96 -83126.38 -69497.99</t>
-  </si>
-  <si>
-    <t>BEV100         -20787.13 -26851.67 -15086.89</t>
-  </si>
-  <si>
-    <t>BEV200         -14923.45 -18796.25 -11304.47</t>
-  </si>
-  <si>
-    <t>BEV300          -9059.78 -11958.09  -6412.11</t>
-  </si>
-  <si>
-    <t>powertrainbev  -19996.42 -26483.38 -13899.11</t>
-  </si>
-  <si>
-    <t>powertrainhev   -1265.50  -2490.90    -90.44</t>
-  </si>
-  <si>
-    <t>range_bev        4150.66   1460.24   6911.95</t>
-  </si>
-  <si>
-    <t>mileage         -1521.86  -1988.61  -1092.73</t>
-  </si>
-  <si>
-    <t>age              -443.37   -687.02   -212.62</t>
-  </si>
-  <si>
-    <t>operating_cost  -5374.86  -7104.17  -3753.86</t>
-  </si>
-  <si>
-    <t>no_choice      -42408.66 -46844.64 -38459.40</t>
-  </si>
-  <si>
-    <t>BEV100         -15845.76 -19855.08 -12180.76</t>
-  </si>
-  <si>
-    <t>BEV200         -11695.10 -14006.70  -9690.49</t>
-  </si>
-  <si>
-    <t>BEV300          -7544.45 -10720.82  -4547.84</t>
-  </si>
-  <si>
     <t>powertrainbev  -26106.06 -33315.10 -20391.86</t>
   </si>
   <si>
@@ -1187,13 +834,355 @@
   </si>
   <si>
     <t>conf_model_suv_int_p_m</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Estimate Std. Error z-value Pr(&gt;|z|) </t>
+  </si>
+  <si>
+    <t>powertrainbev -1.8981055 0.1228924 -15.4453 &lt; 2.2e-16 ***</t>
+  </si>
+  <si>
+    <t xml:space="preserve">powertrainhev -0.1669387 0.0583318 -2.8619 0.004211 ** </t>
+  </si>
+  <si>
+    <t>range_bev 0.5496466 0.0711309 7.7273 1.088e-14 ***</t>
+  </si>
+  <si>
+    <t>mileage -0.2108259 0.0168614 -12.5034 &lt; 2.2e-16 ***</t>
+  </si>
+  <si>
+    <t>age -0.0758603 0.0095932 -7.9077 2.665e-15 ***</t>
+  </si>
+  <si>
+    <t>operating_cost -0.8060906 0.0718606 -11.2174 &lt; 2.2e-16 ***</t>
+  </si>
+  <si>
+    <t>price -0.9486337 0.0393496 -24.1078 &lt; 2.2e-16 ***</t>
+  </si>
+  <si>
+    <t>no_choice -5.2388974 0.1694846 -30.9108 &lt; 2.2e-16 ***</t>
+  </si>
+  <si>
+    <t>Signif. codes: 0 ‘***’ 0.001 ‘**’ 0.01 ‘*’ 0.05 ‘.’ 0.1 ‘ ’ 1</t>
+  </si>
+  <si>
+    <t>Log-Likelihood: -4732.0054845</t>
+  </si>
+  <si>
+    <t>Null Log-Likelihood: -5556.2677994</t>
+  </si>
+  <si>
+    <t>AIC: 9480.0109690</t>
+  </si>
+  <si>
+    <t>BIC: 9530.3794000</t>
+  </si>
+  <si>
+    <t>McFadden R2: 0.1483482</t>
+  </si>
+  <si>
+    <t>Adj McFadden R2: 0.1469084</t>
+  </si>
+  <si>
+    <t>Number of Observations: 4008.0000000</t>
+  </si>
+  <si>
+    <t>powertrainbev -2.5169749 0.1776295 -14.1698 &lt;2e-16 ***</t>
+  </si>
+  <si>
+    <t xml:space="preserve">powertrainhev -0.0223884 0.0495722 -0.4516 0.6515 </t>
+  </si>
+  <si>
+    <t>range_bev 0.5748933 0.0636751 9.0285 &lt;2e-16 ***</t>
+  </si>
+  <si>
+    <t>mileage -0.2454645 0.0167748 -14.6329 &lt;2e-16 ***</t>
+  </si>
+  <si>
+    <t>age -0.1143782 0.0095746 -11.9460 &lt;2e-16 ***</t>
+  </si>
+  <si>
+    <t>operating_cost -0.6104738 0.0635862 -9.6007 &lt;2e-16 ***</t>
+  </si>
+  <si>
+    <t>price -0.7831601 0.0328087 -23.8705 &lt;2e-16 ***</t>
+  </si>
+  <si>
+    <t>no_choice -5.2644607 0.1687681 -31.1935 &lt;2e-16 ***</t>
+  </si>
+  <si>
+    <t>Log-Likelihood: -5222.6778991</t>
+  </si>
+  <si>
+    <t>Null Log-Likelihood: -5955.5205754</t>
+  </si>
+  <si>
+    <t>AIC: 10461.3557982</t>
+  </si>
+  <si>
+    <t>BIC: 10512.2793000</t>
+  </si>
+  <si>
+    <t>McFadden R2: 0.1230527</t>
+  </si>
+  <si>
+    <t>Adj McFadden R2: 0.1217094</t>
+  </si>
+  <si>
+    <t>Number of Observations: 4296.0000000</t>
+  </si>
+  <si>
+    <t>scalePar 2.0997771 0.0917621 22.8828 &lt; 2.2e-16 ***</t>
+  </si>
+  <si>
+    <t>no_choice -3.0892093 0.1062021 -29.0880 &lt; 2.2e-16 ***</t>
+  </si>
+  <si>
+    <t>powertrainbev -0.8282092 0.0857427 -9.6592 &lt; 2.2e-16 ***</t>
+  </si>
+  <si>
+    <t>powertrainhev -0.1461649 0.0367776 -3.9743 7.059e-05 ***</t>
+  </si>
+  <si>
+    <t xml:space="preserve">range_bev 0.0876791 0.0647908 1.3533 0.176 </t>
+  </si>
+  <si>
+    <t>mileage -0.0958517 0.0109261 -8.7727 &lt; 2.2e-16 ***</t>
+  </si>
+  <si>
+    <t>age -0.0236684 0.0060438 -3.9162 8.997e-05 ***</t>
+  </si>
+  <si>
+    <t>operating_cost -0.4307555 0.0468940 -9.1857 &lt; 2.2e-16 ***</t>
+  </si>
+  <si>
+    <t>Log-Likelihood: -2797.1174745</t>
+  </si>
+  <si>
+    <t>Null Log-Likelihood: -3451.8729592</t>
+  </si>
+  <si>
+    <t>AIC: 5610.2349490</t>
+  </si>
+  <si>
+    <t>BIC: 5656.7953000</t>
+  </si>
+  <si>
+    <t>McFadden R2: 0.1896812</t>
+  </si>
+  <si>
+    <t>Adj McFadden R2: 0.1873636</t>
+  </si>
+  <si>
+    <t>Number of Observations: 2490.0000000</t>
+  </si>
+  <si>
+    <t>scalePar 0.882397 0.054098 16.3112 &lt; 2.2e-16 ***</t>
+  </si>
+  <si>
+    <t>no_choice -6.495162 0.322266 -20.1547 &lt; 2.2e-16 ***</t>
+  </si>
+  <si>
+    <t>powertrainbev -1.839372 0.308366 -5.9649 2.448e-09 ***</t>
+  </si>
+  <si>
+    <t xml:space="preserve">powertrainhev 0.083122 0.110104 0.7549 0.4503 </t>
+  </si>
+  <si>
+    <t>range_bev 0.553919 0.140069 3.9546 7.666e-05 ***</t>
+  </si>
+  <si>
+    <t>mileage -0.289556 0.034590 -8.3712 &lt; 2.2e-16 ***</t>
+  </si>
+  <si>
+    <t>age -0.143556 0.019472 -7.3723 1.676e-13 ***</t>
+  </si>
+  <si>
+    <t>operating_cost -0.844735 0.143258 -5.8966 3.711e-09 ***</t>
+  </si>
+  <si>
+    <t>Log-Likelihood: -1782.5764675</t>
+  </si>
+  <si>
+    <t>Null Log-Likelihood: -2104.3948402</t>
+  </si>
+  <si>
+    <t>AIC: 3581.1529350</t>
+  </si>
+  <si>
+    <t>BIC: 3623.7541000</t>
+  </si>
+  <si>
+    <t>McFadden R2: 0.1529268</t>
+  </si>
+  <si>
+    <t>Adj McFadden R2: 0.1491252</t>
+  </si>
+  <si>
+    <t>Number of Observations: 1518.0000000</t>
+  </si>
+  <si>
+    <t>scalePar 1.5851422 0.0892471 17.7613 &lt; 2.2e-16 ***</t>
+  </si>
+  <si>
+    <t>no_choice -3.8984822 0.1603637 -24.3103 &lt; 2.2e-16 ***</t>
+  </si>
+  <si>
+    <t>powertrainbev -1.8525926 0.2436600 -7.6032 2.887e-14 ***</t>
+  </si>
+  <si>
+    <t xml:space="preserve">powertrainhev -0.0965378 0.0492685 -1.9594 0.0500631 . </t>
+  </si>
+  <si>
+    <t>range_bev 0.4212463 0.1079008 3.9040 9.461e-05 ***</t>
+  </si>
+  <si>
+    <t>mileage -0.1297198 0.0179325 -7.2338 4.696e-13 ***</t>
+  </si>
+  <si>
+    <t>age -0.0327588 0.0098211 -3.3356 0.0008513 ***</t>
+  </si>
+  <si>
+    <t>operating_cost -0.4693481 0.0682069 -6.8812 5.933e-12 ***</t>
+  </si>
+  <si>
+    <t>Log-Likelihood: -1939.1128692</t>
+  </si>
+  <si>
+    <t>Null Log-Likelihood: -2312.3389943</t>
+  </si>
+  <si>
+    <t>AIC: 3894.2257384</t>
+  </si>
+  <si>
+    <t>BIC: 3937.5808000</t>
+  </si>
+  <si>
+    <t>McFadden R2: 0.1614063</t>
+  </si>
+  <si>
+    <t>Adj McFadden R2: 0.1579466</t>
+  </si>
+  <si>
+    <t>Number of Observations: 1668.0000000</t>
+  </si>
+  <si>
+    <t>scalePar 0.786014 0.041167 19.0931 &lt; 2.2e-16 ***</t>
+  </si>
+  <si>
+    <t>no_choice -7.259847 0.280427 -25.8885 &lt; 2.2e-16 ***</t>
+  </si>
+  <si>
+    <t>powertrainbev -2.610250 0.359155 -7.2677 3.655e-13 ***</t>
+  </si>
+  <si>
+    <t xml:space="preserve">powertrainhev 0.076302 0.084138 0.9069 0.3645 </t>
+  </si>
+  <si>
+    <t>range_bev 0.549873 0.114029 4.8222 1.420e-06 ***</t>
+  </si>
+  <si>
+    <t>mileage -0.358177 0.032093 -11.1606 &lt; 2.2e-16 ***</t>
+  </si>
+  <si>
+    <t>age -0.203140 0.018267 -11.1203 &lt; 2.2e-16 ***</t>
+  </si>
+  <si>
+    <t>operating_cost -0.710237 0.110088 -6.4515 1.107e-10 ***</t>
+  </si>
+  <si>
+    <t>Log-Likelihood: -3189.5520955</t>
+  </si>
+  <si>
+    <t>Null Log-Likelihood: -3643.1815810</t>
+  </si>
+  <si>
+    <t>AIC: 6395.1041910</t>
+  </si>
+  <si>
+    <t>BIC: 6442.0960000</t>
+  </si>
+  <si>
+    <t>McFadden R2: 0.1245147</t>
+  </si>
+  <si>
+    <t>Adj McFadden R2: 0.1223188</t>
+  </si>
+  <si>
+    <t>Number of Observations: 2628.0000000</t>
+  </si>
+  <si>
+    <t>Variable</t>
+  </si>
+  <si>
+    <t>mean</t>
+  </si>
+  <si>
+    <t>lower</t>
+  </si>
+  <si>
+    <t>upper</t>
+  </si>
+  <si>
+    <t>powertrainbev</t>
+  </si>
+  <si>
+    <t>powertrainhev</t>
+  </si>
+  <si>
+    <t>range_bev</t>
+  </si>
+  <si>
+    <t>mileage</t>
+  </si>
+  <si>
+    <t>age</t>
+  </si>
+  <si>
+    <t>operating_cost</t>
+  </si>
+  <si>
+    <t>price</t>
+  </si>
+  <si>
+    <t>no_choice</t>
+  </si>
+  <si>
+    <t>BEV100</t>
+  </si>
+  <si>
+    <t>BEV200</t>
+  </si>
+  <si>
+    <t>BEV300</t>
+  </si>
+  <si>
+    <t>Mean</t>
+  </si>
+  <si>
+    <t>Lower</t>
+  </si>
+  <si>
+    <t>Upper</t>
+  </si>
+  <si>
+    <t>model_positive_group_car</t>
+  </si>
+  <si>
+    <t>model_negative_group_car</t>
+  </si>
+  <si>
+    <t>model_positive_group_suv</t>
+  </si>
+  <si>
+    <t>model_negative_group_suv</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1214,8 +1203,22 @@
       <name val="Lucida Console"/>
       <family val="3"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3B3B3B"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1228,8 +1231,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -1237,11 +1246,26 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1254,6 +1278,60 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1598,176 +1676,172 @@
   <sheetData>
     <row r="2" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B2" s="3" t="s">
-        <v>89</v>
+        <v>24</v>
       </c>
       <c r="C2" s="4"/>
       <c r="D2" s="4"/>
       <c r="E2" s="4"/>
       <c r="F2" s="4"/>
       <c r="G2" s="3" t="s">
-        <v>90</v>
+        <v>25</v>
       </c>
       <c r="H2" s="4"/>
     </row>
     <row r="3" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B3" s="1" t="s">
+      <c r="B3" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="G3" s="1" t="s">
+      <c r="G3" s="5" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="4" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B4" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="G4" s="1" t="s">
-        <v>91</v>
+      <c r="B4" s="5" t="s">
+        <v>264</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>264</v>
       </c>
     </row>
     <row r="5" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B5" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="G5" s="1" t="s">
-        <v>92</v>
+      <c r="B5" s="5" t="s">
+        <v>265</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>281</v>
       </c>
     </row>
     <row r="6" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B6" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="G6" s="1" t="s">
-        <v>93</v>
+      <c r="B6" s="5" t="s">
+        <v>266</v>
+      </c>
+      <c r="G6" s="5" t="s">
+        <v>282</v>
       </c>
     </row>
     <row r="7" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B7" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="G7" s="1" t="s">
-        <v>94</v>
+      <c r="B7" s="5" t="s">
+        <v>267</v>
+      </c>
+      <c r="G7" s="5" t="s">
+        <v>283</v>
       </c>
     </row>
     <row r="8" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B8" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="G8" s="1" t="s">
-        <v>95</v>
+      <c r="B8" s="5" t="s">
+        <v>268</v>
+      </c>
+      <c r="G8" s="5" t="s">
+        <v>284</v>
       </c>
     </row>
     <row r="9" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B9" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="G9" s="1" t="s">
-        <v>96</v>
+      <c r="B9" s="5" t="s">
+        <v>269</v>
+      </c>
+      <c r="G9" s="5" t="s">
+        <v>285</v>
       </c>
     </row>
     <row r="10" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B10" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="G10" s="1" t="s">
-        <v>97</v>
+      <c r="B10" s="5" t="s">
+        <v>270</v>
+      </c>
+      <c r="G10" s="5" t="s">
+        <v>286</v>
       </c>
     </row>
     <row r="11" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B11" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="G11" s="1" t="s">
-        <v>98</v>
+      <c r="B11" s="5" t="s">
+        <v>271</v>
+      </c>
+      <c r="G11" s="5" t="s">
+        <v>287</v>
       </c>
     </row>
     <row r="12" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B12" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="G12" s="1" t="s">
-        <v>99</v>
+      <c r="B12" s="5" t="s">
+        <v>272</v>
+      </c>
+      <c r="G12" s="5" t="s">
+        <v>288</v>
       </c>
     </row>
     <row r="13" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B13" s="1" t="s">
+      <c r="B13" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="G13" s="1" t="s">
+      <c r="G13" s="5" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="14" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B14" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="G14" s="1" t="s">
-        <v>3</v>
+      <c r="B14" s="5" t="s">
+        <v>273</v>
+      </c>
+      <c r="G14" s="5" t="s">
+        <v>273</v>
       </c>
     </row>
     <row r="15" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B15" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="G15" s="1" t="s">
-        <v>4</v>
+      <c r="B15" s="5" t="s">
+        <v>274</v>
+      </c>
+      <c r="G15" s="5" t="s">
+        <v>289</v>
       </c>
     </row>
     <row r="16" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B16" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="G16" s="1" t="s">
-        <v>100</v>
+      <c r="B16" s="5" t="s">
+        <v>275</v>
+      </c>
+      <c r="G16" s="5" t="s">
+        <v>290</v>
       </c>
     </row>
     <row r="17" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B17" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="G17" s="1" t="s">
-        <v>101</v>
+      <c r="B17" s="5" t="s">
+        <v>276</v>
+      </c>
+      <c r="G17" s="5" t="s">
+        <v>291</v>
       </c>
     </row>
     <row r="18" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B18" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="G18" s="1" t="s">
-        <v>102</v>
+      <c r="B18" s="5" t="s">
+        <v>277</v>
+      </c>
+      <c r="G18" s="5" t="s">
+        <v>292</v>
       </c>
     </row>
     <row r="19" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B19" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="G19" s="1" t="s">
-        <v>103</v>
+      <c r="B19" s="5" t="s">
+        <v>278</v>
+      </c>
+      <c r="G19" s="5" t="s">
+        <v>293</v>
       </c>
     </row>
     <row r="20" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B20" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="G20" s="1" t="s">
-        <v>104</v>
+      <c r="B20" s="5" t="s">
+        <v>279</v>
+      </c>
+      <c r="G20" s="5" t="s">
+        <v>294</v>
       </c>
     </row>
     <row r="21" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B21" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="G21" s="1" t="s">
-        <v>105</v>
+      <c r="B21" s="5" t="s">
+        <v>280</v>
+      </c>
+      <c r="G21" s="5" t="s">
+        <v>295</v>
       </c>
     </row>
     <row r="22" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B22" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="G22" s="2" t="s">
-        <v>106</v>
-      </c>
+      <c r="B22" s="2"/>
+      <c r="G22" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1776,7 +1850,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{059E5AF4-7A4F-4492-8136-3B99EF90548D}">
-  <dimension ref="B2:F45"/>
+  <dimension ref="B2:F44"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="81.5703125" bestFit="1" customWidth="1"/>
@@ -1792,164 +1866,160 @@
       </c>
     </row>
     <row r="3" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B3" s="1" t="s">
+      <c r="B3" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="F3" s="1" t="s">
+      <c r="F3" s="5" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="4" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B4" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>1</v>
+      <c r="B4" s="5" t="s">
+        <v>264</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>264</v>
       </c>
     </row>
     <row r="5" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B5" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="F5" s="1" t="s">
-        <v>44</v>
+      <c r="B5" s="5" t="s">
+        <v>296</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>326</v>
       </c>
     </row>
     <row r="6" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B6" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="F6" s="1" t="s">
-        <v>45</v>
+      <c r="B6" s="5" t="s">
+        <v>297</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>327</v>
       </c>
     </row>
     <row r="7" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B7" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="F7" s="1" t="s">
-        <v>46</v>
+      <c r="B7" s="5" t="s">
+        <v>298</v>
+      </c>
+      <c r="F7" s="5" t="s">
+        <v>328</v>
       </c>
     </row>
     <row r="8" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B8" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="F8" s="1" t="s">
-        <v>47</v>
+      <c r="B8" s="5" t="s">
+        <v>299</v>
+      </c>
+      <c r="F8" s="5" t="s">
+        <v>329</v>
       </c>
     </row>
     <row r="9" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B9" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="F9" s="1" t="s">
-        <v>48</v>
+      <c r="B9" s="5" t="s">
+        <v>300</v>
+      </c>
+      <c r="F9" s="5" t="s">
+        <v>330</v>
       </c>
     </row>
     <row r="10" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B10" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="F10" s="1" t="s">
-        <v>49</v>
+      <c r="B10" s="5" t="s">
+        <v>301</v>
+      </c>
+      <c r="F10" s="5" t="s">
+        <v>331</v>
       </c>
     </row>
     <row r="11" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B11" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="F11" s="1" t="s">
-        <v>50</v>
+      <c r="B11" s="5" t="s">
+        <v>302</v>
+      </c>
+      <c r="F11" s="5" t="s">
+        <v>332</v>
       </c>
     </row>
     <row r="12" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B12" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="F12" s="1" t="s">
-        <v>51</v>
+      <c r="B12" s="5" t="s">
+        <v>303</v>
+      </c>
+      <c r="F12" s="5" t="s">
+        <v>333</v>
       </c>
     </row>
     <row r="13" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B13" s="1" t="s">
+      <c r="B13" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="F13" s="1" t="s">
+      <c r="F13" s="5" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="14" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B14" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="F14" s="1" t="s">
-        <v>3</v>
+      <c r="B14" s="5" t="s">
+        <v>273</v>
+      </c>
+      <c r="F14" s="5" t="s">
+        <v>273</v>
       </c>
     </row>
     <row r="15" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B15" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F15" s="1" t="s">
-        <v>4</v>
+      <c r="B15" s="5" t="s">
+        <v>304</v>
+      </c>
+      <c r="F15" s="5" t="s">
+        <v>334</v>
       </c>
     </row>
     <row r="16" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B16" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="F16" s="1" t="s">
-        <v>52</v>
+      <c r="B16" s="5" t="s">
+        <v>305</v>
+      </c>
+      <c r="F16" s="5" t="s">
+        <v>335</v>
       </c>
     </row>
     <row r="17" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B17" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="F17" s="1" t="s">
-        <v>53</v>
+      <c r="B17" s="5" t="s">
+        <v>306</v>
+      </c>
+      <c r="F17" s="5" t="s">
+        <v>336</v>
       </c>
     </row>
     <row r="18" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B18" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="F18" s="1" t="s">
-        <v>54</v>
+      <c r="B18" s="5" t="s">
+        <v>307</v>
+      </c>
+      <c r="F18" s="5" t="s">
+        <v>337</v>
       </c>
     </row>
     <row r="19" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B19" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="F19" s="1" t="s">
-        <v>55</v>
+      <c r="B19" s="5" t="s">
+        <v>308</v>
+      </c>
+      <c r="F19" s="5" t="s">
+        <v>338</v>
       </c>
     </row>
     <row r="20" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B20" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="F20" s="1" t="s">
-        <v>56</v>
+      <c r="B20" s="5" t="s">
+        <v>309</v>
+      </c>
+      <c r="F20" s="5" t="s">
+        <v>339</v>
       </c>
     </row>
     <row r="21" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B21" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="F21" s="1" t="s">
-        <v>57</v>
+      <c r="B21" s="5" t="s">
+        <v>310</v>
+      </c>
+      <c r="F21" s="5" t="s">
+        <v>340</v>
       </c>
     </row>
     <row r="22" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B22" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="F22" s="2" t="s">
-        <v>58</v>
-      </c>
+      <c r="B22" s="2"/>
+      <c r="F22" s="2"/>
     </row>
     <row r="25" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B25" s="3" t="s">
@@ -1960,163 +2030,155 @@
       </c>
     </row>
     <row r="26" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B26" s="1" t="s">
+      <c r="B26" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="F26" s="1" t="s">
+      <c r="F26" s="5" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="27" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B27" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="F27" s="1" t="s">
-        <v>1</v>
+      <c r="B27" s="5" t="s">
+        <v>264</v>
+      </c>
+      <c r="F27" s="5" t="s">
+        <v>264</v>
       </c>
     </row>
     <row r="28" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B28" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="F28" s="1" t="s">
-        <v>59</v>
+      <c r="B28" s="5" t="s">
+        <v>311</v>
+      </c>
+      <c r="F28" s="5" t="s">
+        <v>341</v>
       </c>
     </row>
     <row r="29" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B29" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="F29" s="1" t="s">
-        <v>60</v>
+      <c r="B29" s="5" t="s">
+        <v>312</v>
+      </c>
+      <c r="F29" s="5" t="s">
+        <v>342</v>
       </c>
     </row>
     <row r="30" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B30" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="F30" s="1" t="s">
-        <v>61</v>
+      <c r="B30" s="5" t="s">
+        <v>313</v>
+      </c>
+      <c r="F30" s="5" t="s">
+        <v>343</v>
       </c>
     </row>
     <row r="31" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B31" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="F31" s="1" t="s">
-        <v>62</v>
+      <c r="B31" s="5" t="s">
+        <v>314</v>
+      </c>
+      <c r="F31" s="5" t="s">
+        <v>344</v>
       </c>
     </row>
     <row r="32" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B32" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="F32" s="1" t="s">
-        <v>63</v>
+      <c r="B32" s="5" t="s">
+        <v>315</v>
+      </c>
+      <c r="F32" s="5" t="s">
+        <v>345</v>
       </c>
     </row>
     <row r="33" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B33" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="F33" s="1" t="s">
-        <v>64</v>
+      <c r="B33" s="5" t="s">
+        <v>316</v>
+      </c>
+      <c r="F33" s="5" t="s">
+        <v>346</v>
       </c>
     </row>
     <row r="34" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B34" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="F34" s="1" t="s">
-        <v>65</v>
+      <c r="B34" s="5" t="s">
+        <v>317</v>
+      </c>
+      <c r="F34" s="5" t="s">
+        <v>347</v>
       </c>
     </row>
     <row r="35" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B35" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="F35" s="1" t="s">
-        <v>66</v>
+      <c r="B35" s="5" t="s">
+        <v>318</v>
+      </c>
+      <c r="F35" s="5" t="s">
+        <v>348</v>
       </c>
     </row>
     <row r="36" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B36" s="1" t="s">
+      <c r="B36" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="F36" s="1" t="s">
+      <c r="F36" s="5" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="37" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B37" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="F37" s="1" t="s">
-        <v>3</v>
+      <c r="B37" s="5" t="s">
+        <v>273</v>
+      </c>
+      <c r="F37" s="5" t="s">
+        <v>273</v>
       </c>
     </row>
     <row r="38" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B38" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F38" s="1" t="s">
-        <v>4</v>
+      <c r="B38" s="5" t="s">
+        <v>319</v>
+      </c>
+      <c r="F38" s="5" t="s">
+        <v>349</v>
       </c>
     </row>
     <row r="39" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B39" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="F39" s="1" t="s">
-        <v>67</v>
+      <c r="B39" s="5" t="s">
+        <v>320</v>
+      </c>
+      <c r="F39" s="5" t="s">
+        <v>350</v>
       </c>
     </row>
     <row r="40" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B40" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="F40" s="1" t="s">
-        <v>68</v>
+      <c r="B40" s="5" t="s">
+        <v>321</v>
+      </c>
+      <c r="F40" s="5" t="s">
+        <v>351</v>
       </c>
     </row>
     <row r="41" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B41" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="F41" s="1" t="s">
-        <v>69</v>
+      <c r="B41" s="5" t="s">
+        <v>322</v>
+      </c>
+      <c r="F41" s="5" t="s">
+        <v>352</v>
       </c>
     </row>
     <row r="42" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B42" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="F42" s="1" t="s">
-        <v>70</v>
+      <c r="B42" s="5" t="s">
+        <v>323</v>
+      </c>
+      <c r="F42" s="5" t="s">
+        <v>353</v>
       </c>
     </row>
     <row r="43" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B43" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="F43" s="1" t="s">
-        <v>71</v>
+      <c r="B43" s="5" t="s">
+        <v>324</v>
+      </c>
+      <c r="F43" s="5" t="s">
+        <v>354</v>
       </c>
     </row>
     <row r="44" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B44" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="F44" s="1" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="45" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B45" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="F45" s="2" t="s">
-        <v>73</v>
+      <c r="B44" s="5" t="s">
+        <v>325</v>
+      </c>
+      <c r="F44" s="5" t="s">
+        <v>355</v>
       </c>
     </row>
   </sheetData>
@@ -2126,227 +2188,1377 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EBB0F02F-467D-4060-A25E-228F81E04657}">
-  <dimension ref="C2:G30"/>
+  <dimension ref="C2:M30"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="3" max="3" width="61" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="61" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="29.5703125" customWidth="1"/>
+    <col min="8" max="8" width="21.85546875" customWidth="1"/>
+    <col min="10" max="10" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C2" s="3" t="s">
+    <row r="2" spans="3:13" x14ac:dyDescent="0.25">
+      <c r="C2" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="D2" s="14"/>
+      <c r="E2" s="14"/>
+      <c r="F2" s="14"/>
+      <c r="H2" s="14" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="3" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C3" s="1" t="s">
-        <v>282</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>282</v>
-      </c>
-    </row>
-    <row r="4" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C4" s="1" t="s">
-        <v>283</v>
-      </c>
-      <c r="G4" s="1" t="s">
-        <v>314</v>
-      </c>
-    </row>
-    <row r="5" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C5" s="1" t="s">
-        <v>284</v>
-      </c>
-      <c r="G5" s="1" t="s">
-        <v>315</v>
-      </c>
-    </row>
-    <row r="6" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C6" s="1" t="s">
-        <v>285</v>
-      </c>
-      <c r="G6" s="1" t="s">
-        <v>316</v>
-      </c>
-    </row>
-    <row r="7" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C7" s="1" t="s">
-        <v>286</v>
-      </c>
-      <c r="G7" s="1" t="s">
-        <v>317</v>
-      </c>
-    </row>
-    <row r="8" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C8" s="1" t="s">
-        <v>287</v>
-      </c>
-      <c r="G8" s="1" t="s">
-        <v>318</v>
-      </c>
-    </row>
-    <row r="9" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C9" s="1" t="s">
-        <v>288</v>
-      </c>
-      <c r="G9" s="1" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="10" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C10" s="1" t="s">
-        <v>289</v>
-      </c>
-      <c r="G10" s="1" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="11" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C11" s="1" t="s">
-        <v>290</v>
-      </c>
-      <c r="G11" s="1" t="s">
-        <v>320</v>
-      </c>
-    </row>
-    <row r="12" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C12" s="1" t="s">
-        <v>291</v>
-      </c>
-      <c r="G12" s="1" t="s">
-        <v>321</v>
-      </c>
-    </row>
-    <row r="13" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C13" s="1" t="s">
-        <v>292</v>
-      </c>
-      <c r="G13" s="1" t="s">
-        <v>322</v>
-      </c>
-    </row>
-    <row r="14" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C14" s="2" t="s">
-        <v>293</v>
-      </c>
-      <c r="G14" s="2" t="s">
-        <v>323</v>
-      </c>
-    </row>
-    <row r="18" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C18" s="3" t="s">
+      <c r="I2" s="14"/>
+      <c r="J2" s="14"/>
+      <c r="K2" s="14"/>
+    </row>
+    <row r="3" spans="3:13" x14ac:dyDescent="0.25">
+      <c r="C3" s="8" t="s">
+        <v>356</v>
+      </c>
+      <c r="D3" s="9" t="s">
+        <v>357</v>
+      </c>
+      <c r="E3" s="9" t="s">
+        <v>358</v>
+      </c>
+      <c r="F3" s="9" t="s">
+        <v>359</v>
+      </c>
+      <c r="H3" s="8" t="s">
+        <v>356</v>
+      </c>
+      <c r="I3" s="9" t="s">
+        <v>357</v>
+      </c>
+      <c r="J3" s="9" t="s">
+        <v>358</v>
+      </c>
+      <c r="K3" s="9" t="s">
+        <v>359</v>
+      </c>
+      <c r="L3" s="7"/>
+      <c r="M3" s="7"/>
+    </row>
+    <row r="4" spans="3:13" x14ac:dyDescent="0.25">
+      <c r="C4" s="10" t="s">
+        <v>360</v>
+      </c>
+      <c r="D4" s="11">
+        <v>-8296.65</v>
+      </c>
+      <c r="E4" s="11">
+        <v>-10043</v>
+      </c>
+      <c r="F4" s="11">
+        <v>-6618.42</v>
+      </c>
+      <c r="H4" s="10" t="s">
+        <v>360</v>
+      </c>
+      <c r="I4" s="11">
+        <v>-18587.740000000002</v>
+      </c>
+      <c r="J4" s="11">
+        <v>-23514.12</v>
+      </c>
+      <c r="K4" s="11">
+        <v>-13846.7</v>
+      </c>
+      <c r="L4" s="6"/>
+      <c r="M4" s="6"/>
+    </row>
+    <row r="5" spans="3:13" x14ac:dyDescent="0.25">
+      <c r="C5" s="10" t="s">
+        <v>361</v>
+      </c>
+      <c r="D5" s="11">
+        <v>-1461.24</v>
+      </c>
+      <c r="E5" s="11">
+        <v>-2185.9699999999998</v>
+      </c>
+      <c r="F5" s="11">
+        <v>-752.91</v>
+      </c>
+      <c r="H5" s="10" t="s">
+        <v>361</v>
+      </c>
+      <c r="I5" s="11">
+        <v>-964.48</v>
+      </c>
+      <c r="J5" s="11">
+        <v>-1963.2</v>
+      </c>
+      <c r="K5" s="11">
+        <v>12.17</v>
+      </c>
+      <c r="L5" s="6"/>
+      <c r="M5" s="6"/>
+    </row>
+    <row r="6" spans="3:13" x14ac:dyDescent="0.25">
+      <c r="C6" s="10" t="s">
+        <v>362</v>
+      </c>
+      <c r="D6" s="11">
+        <v>878.24</v>
+      </c>
+      <c r="E6" s="11">
+        <v>-393.23</v>
+      </c>
+      <c r="F6" s="11">
+        <v>2164.09</v>
+      </c>
+      <c r="H6" s="10" t="s">
+        <v>362</v>
+      </c>
+      <c r="I6" s="11">
+        <v>4229.0200000000004</v>
+      </c>
+      <c r="J6" s="11">
+        <v>2119.0700000000002</v>
+      </c>
+      <c r="K6" s="11">
+        <v>6339.29</v>
+      </c>
+      <c r="L6" s="6"/>
+      <c r="M6" s="6"/>
+    </row>
+    <row r="7" spans="3:13" x14ac:dyDescent="0.25">
+      <c r="C7" s="10" t="s">
+        <v>363</v>
+      </c>
+      <c r="D7" s="11">
+        <v>-960.62</v>
+      </c>
+      <c r="E7" s="11">
+        <v>-1182.01</v>
+      </c>
+      <c r="F7" s="11">
+        <v>-751.82</v>
+      </c>
+      <c r="H7" s="10" t="s">
+        <v>363</v>
+      </c>
+      <c r="I7" s="11">
+        <v>-1298.97</v>
+      </c>
+      <c r="J7" s="11">
+        <v>-1670.53</v>
+      </c>
+      <c r="K7" s="11">
+        <v>-953.72</v>
+      </c>
+      <c r="L7" s="6"/>
+      <c r="M7" s="6"/>
+    </row>
+    <row r="8" spans="3:13" x14ac:dyDescent="0.25">
+      <c r="C8" s="10" t="s">
+        <v>364</v>
+      </c>
+      <c r="D8" s="11">
+        <v>-236.89</v>
+      </c>
+      <c r="E8" s="11">
+        <v>-356.49</v>
+      </c>
+      <c r="F8" s="11">
+        <v>-120.17</v>
+      </c>
+      <c r="H8" s="10" t="s">
+        <v>364</v>
+      </c>
+      <c r="I8" s="11">
+        <v>-329.12</v>
+      </c>
+      <c r="J8" s="11">
+        <v>-522.92999999999995</v>
+      </c>
+      <c r="K8" s="11">
+        <v>-137.97</v>
+      </c>
+      <c r="L8" s="6"/>
+      <c r="M8" s="6"/>
+    </row>
+    <row r="9" spans="3:13" x14ac:dyDescent="0.25">
+      <c r="C9" s="10" t="s">
+        <v>365</v>
+      </c>
+      <c r="D9" s="11">
+        <v>-4309.71</v>
+      </c>
+      <c r="E9" s="11">
+        <v>-5250.3</v>
+      </c>
+      <c r="F9" s="11">
+        <v>-3404.5</v>
+      </c>
+      <c r="H9" s="10" t="s">
+        <v>365</v>
+      </c>
+      <c r="I9" s="11">
+        <v>-4712.09</v>
+      </c>
+      <c r="J9" s="11">
+        <v>-6113.02</v>
+      </c>
+      <c r="K9" s="11">
+        <v>-3382.97</v>
+      </c>
+      <c r="L9" s="6"/>
+      <c r="M9" s="6"/>
+    </row>
+    <row r="10" spans="3:13" x14ac:dyDescent="0.25">
+      <c r="C10" s="10" t="s">
+        <v>366</v>
+      </c>
+      <c r="D10" s="11">
+        <v>-10000</v>
+      </c>
+      <c r="E10" s="11">
+        <v>-10000</v>
+      </c>
+      <c r="F10" s="11">
+        <v>-10000</v>
+      </c>
+      <c r="H10" s="10" t="s">
+        <v>366</v>
+      </c>
+      <c r="I10" s="11">
+        <v>-10000</v>
+      </c>
+      <c r="J10" s="11">
+        <v>-10000</v>
+      </c>
+      <c r="K10" s="11">
+        <v>-10000</v>
+      </c>
+      <c r="L10" s="6"/>
+      <c r="M10" s="6"/>
+    </row>
+    <row r="11" spans="3:13" x14ac:dyDescent="0.25">
+      <c r="C11" s="10" t="s">
+        <v>367</v>
+      </c>
+      <c r="D11" s="11">
+        <v>-30919.16</v>
+      </c>
+      <c r="E11" s="11">
+        <v>-33128.83</v>
+      </c>
+      <c r="F11" s="11">
+        <v>-28921.75</v>
+      </c>
+      <c r="H11" s="10" t="s">
+        <v>367</v>
+      </c>
+      <c r="I11" s="11">
+        <v>-39048.370000000003</v>
+      </c>
+      <c r="J11" s="11">
+        <v>-42365.38</v>
+      </c>
+      <c r="K11" s="11">
+        <v>-35950.71</v>
+      </c>
+      <c r="L11" s="6"/>
+      <c r="M11" s="6"/>
+    </row>
+    <row r="12" spans="3:13" x14ac:dyDescent="0.25">
+      <c r="C12" s="12" t="s">
+        <v>368</v>
+      </c>
+      <c r="D12" s="13">
+        <v>-7418.4</v>
+      </c>
+      <c r="E12" s="13">
+        <v>-8462.06</v>
+      </c>
+      <c r="F12" s="13">
+        <v>-6450.67</v>
+      </c>
+      <c r="H12" s="12" t="s">
+        <v>368</v>
+      </c>
+      <c r="I12" s="13">
+        <v>-14358.72</v>
+      </c>
+      <c r="J12" s="13">
+        <v>-17374.84</v>
+      </c>
+      <c r="K12" s="13">
+        <v>-11564.16</v>
+      </c>
+      <c r="L12" s="6"/>
+      <c r="M12" s="6"/>
+    </row>
+    <row r="13" spans="3:13" x14ac:dyDescent="0.25">
+      <c r="C13" s="12" t="s">
+        <v>369</v>
+      </c>
+      <c r="D13" s="13">
+        <v>-6540.16</v>
+      </c>
+      <c r="E13" s="13">
+        <v>-8147.82</v>
+      </c>
+      <c r="F13" s="13">
+        <v>-5016.03</v>
+      </c>
+      <c r="H13" s="12" t="s">
+        <v>369</v>
+      </c>
+      <c r="I13" s="13">
+        <v>-10129.69</v>
+      </c>
+      <c r="J13" s="13">
+        <v>-11804.28</v>
+      </c>
+      <c r="K13" s="13">
+        <v>-8570.0400000000009</v>
+      </c>
+      <c r="L13" s="6"/>
+      <c r="M13" s="6"/>
+    </row>
+    <row r="14" spans="3:13" x14ac:dyDescent="0.25">
+      <c r="C14" s="12" t="s">
+        <v>370</v>
+      </c>
+      <c r="D14" s="13">
+        <v>-5661.92</v>
+      </c>
+      <c r="E14" s="13">
+        <v>-8401.2800000000007</v>
+      </c>
+      <c r="F14" s="13">
+        <v>-2985.22</v>
+      </c>
+      <c r="H14" s="12" t="s">
+        <v>370</v>
+      </c>
+      <c r="I14" s="13">
+        <v>-5900.67</v>
+      </c>
+      <c r="J14" s="13">
+        <v>-8370.7199999999993</v>
+      </c>
+      <c r="K14" s="13">
+        <v>-3540.29</v>
+      </c>
+      <c r="L14" s="6"/>
+      <c r="M14" s="6"/>
+    </row>
+    <row r="18" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C18" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="G18" s="3" t="s">
+      <c r="D18" s="14"/>
+      <c r="E18" s="14"/>
+      <c r="F18" s="14"/>
+      <c r="H18" s="14" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="19" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C19" s="1" t="s">
-        <v>282</v>
-      </c>
-      <c r="G19" s="1" t="s">
-        <v>282</v>
-      </c>
-    </row>
-    <row r="20" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C20" s="1" t="s">
-        <v>294</v>
-      </c>
-      <c r="G20" s="1" t="s">
-        <v>304</v>
-      </c>
-    </row>
-    <row r="21" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C21" s="1" t="s">
-        <v>295</v>
-      </c>
-      <c r="G21" s="1" t="s">
-        <v>305</v>
-      </c>
-    </row>
-    <row r="22" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C22" s="1" t="s">
-        <v>296</v>
-      </c>
-      <c r="G22" s="1" t="s">
-        <v>306</v>
-      </c>
-    </row>
-    <row r="23" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C23" s="1" t="s">
-        <v>297</v>
-      </c>
-      <c r="G23" s="1" t="s">
-        <v>307</v>
-      </c>
-    </row>
-    <row r="24" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C24" s="1" t="s">
-        <v>298</v>
-      </c>
-      <c r="G24" s="1" t="s">
-        <v>308</v>
-      </c>
-    </row>
-    <row r="25" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C25" s="1" t="s">
-        <v>299</v>
-      </c>
-      <c r="G25" s="1" t="s">
-        <v>309</v>
-      </c>
-    </row>
-    <row r="26" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C26" s="1" t="s">
-        <v>289</v>
-      </c>
-      <c r="G26" s="1" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="27" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C27" s="1" t="s">
-        <v>300</v>
-      </c>
-      <c r="G27" s="1" t="s">
-        <v>310</v>
-      </c>
-    </row>
-    <row r="28" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C28" s="1" t="s">
-        <v>301</v>
-      </c>
-      <c r="G28" s="1" t="s">
-        <v>311</v>
-      </c>
-    </row>
-    <row r="29" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C29" s="1" t="s">
-        <v>302</v>
-      </c>
-      <c r="G29" s="1" t="s">
-        <v>312</v>
-      </c>
-    </row>
-    <row r="30" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C30" s="2" t="s">
-        <v>303</v>
-      </c>
-      <c r="G30" s="2" t="s">
-        <v>313</v>
+      <c r="I18" s="14"/>
+      <c r="J18" s="14"/>
+      <c r="K18" s="14"/>
+    </row>
+    <row r="19" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C19" s="8" t="s">
+        <v>356</v>
+      </c>
+      <c r="D19" s="9" t="s">
+        <v>357</v>
+      </c>
+      <c r="E19" s="9" t="s">
+        <v>358</v>
+      </c>
+      <c r="F19" s="9" t="s">
+        <v>359</v>
+      </c>
+      <c r="H19" s="8" t="s">
+        <v>356</v>
+      </c>
+      <c r="I19" s="9" t="s">
+        <v>357</v>
+      </c>
+      <c r="J19" s="9" t="s">
+        <v>358</v>
+      </c>
+      <c r="K19" s="9" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="20" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C20" s="10" t="s">
+        <v>360</v>
+      </c>
+      <c r="D20" s="11">
+        <v>-18478.96</v>
+      </c>
+      <c r="E20" s="11">
+        <v>-24681.48</v>
+      </c>
+      <c r="F20" s="11">
+        <v>-12587.54</v>
+      </c>
+      <c r="H20" s="10" t="s">
+        <v>360</v>
+      </c>
+      <c r="I20" s="11">
+        <v>-26193.86</v>
+      </c>
+      <c r="J20" s="11">
+        <v>-33553.089999999997</v>
+      </c>
+      <c r="K20" s="11">
+        <v>-19307.41</v>
+      </c>
+    </row>
+    <row r="21" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C21" s="10" t="s">
+        <v>361</v>
+      </c>
+      <c r="D21" s="11">
+        <v>825.54</v>
+      </c>
+      <c r="E21" s="11">
+        <v>-1379.43</v>
+      </c>
+      <c r="F21" s="11">
+        <v>3009.8</v>
+      </c>
+      <c r="H21" s="10" t="s">
+        <v>361</v>
+      </c>
+      <c r="I21" s="11">
+        <v>764.08</v>
+      </c>
+      <c r="J21" s="11">
+        <v>-921.12</v>
+      </c>
+      <c r="K21" s="11">
+        <v>2483.98</v>
+      </c>
+    </row>
+    <row r="22" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C22" s="10" t="s">
+        <v>362</v>
+      </c>
+      <c r="D22" s="11">
+        <v>5574.59</v>
+      </c>
+      <c r="E22" s="11">
+        <v>2848.35</v>
+      </c>
+      <c r="F22" s="11">
+        <v>8389.8799999999992</v>
+      </c>
+      <c r="H22" s="10" t="s">
+        <v>362</v>
+      </c>
+      <c r="I22" s="11">
+        <v>5515.55</v>
+      </c>
+      <c r="J22" s="11">
+        <v>3277.32</v>
+      </c>
+      <c r="K22" s="11">
+        <v>7856.52</v>
+      </c>
+    </row>
+    <row r="23" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C23" s="10" t="s">
+        <v>363</v>
+      </c>
+      <c r="D23" s="11">
+        <v>-2902.72</v>
+      </c>
+      <c r="E23" s="11">
+        <v>-3605.09</v>
+      </c>
+      <c r="F23" s="11">
+        <v>-2244.65</v>
+      </c>
+      <c r="H23" s="10" t="s">
+        <v>363</v>
+      </c>
+      <c r="I23" s="11">
+        <v>-3596.63</v>
+      </c>
+      <c r="J23" s="11">
+        <v>-4266.83</v>
+      </c>
+      <c r="K23" s="11">
+        <v>-2983.37</v>
+      </c>
+    </row>
+    <row r="24" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C24" s="10" t="s">
+        <v>364</v>
+      </c>
+      <c r="D24" s="11">
+        <v>-1434.13</v>
+      </c>
+      <c r="E24" s="11">
+        <v>-1836.05</v>
+      </c>
+      <c r="F24" s="11">
+        <v>-1058.5899999999999</v>
+      </c>
+      <c r="H24" s="10" t="s">
+        <v>364</v>
+      </c>
+      <c r="I24" s="11">
+        <v>-2034.68</v>
+      </c>
+      <c r="J24" s="11">
+        <v>-2408.4899999999998</v>
+      </c>
+      <c r="K24" s="11">
+        <v>-1687.69</v>
+      </c>
+    </row>
+    <row r="25" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C25" s="10" t="s">
+        <v>365</v>
+      </c>
+      <c r="D25" s="11">
+        <v>-8465.9</v>
+      </c>
+      <c r="E25" s="11">
+        <v>-11316.64</v>
+      </c>
+      <c r="F25" s="11">
+        <v>-5687.27</v>
+      </c>
+      <c r="H25" s="10" t="s">
+        <v>365</v>
+      </c>
+      <c r="I25" s="11">
+        <v>-7126.64</v>
+      </c>
+      <c r="J25" s="11">
+        <v>-9344.57</v>
+      </c>
+      <c r="K25" s="11">
+        <v>-5031.54</v>
+      </c>
+    </row>
+    <row r="26" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C26" s="10" t="s">
+        <v>366</v>
+      </c>
+      <c r="D26" s="11">
+        <v>-10000</v>
+      </c>
+      <c r="E26" s="11">
+        <v>-10000</v>
+      </c>
+      <c r="F26" s="11">
+        <v>-10000</v>
+      </c>
+      <c r="H26" s="10" t="s">
+        <v>366</v>
+      </c>
+      <c r="I26" s="11">
+        <v>-10000</v>
+      </c>
+      <c r="J26" s="11">
+        <v>-10000</v>
+      </c>
+      <c r="K26" s="11">
+        <v>-10000</v>
+      </c>
+    </row>
+    <row r="27" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C27" s="10" t="s">
+        <v>367</v>
+      </c>
+      <c r="D27" s="11">
+        <v>-65036.95</v>
+      </c>
+      <c r="E27" s="11">
+        <v>-71733.960000000006</v>
+      </c>
+      <c r="F27" s="11">
+        <v>-59032.61</v>
+      </c>
+      <c r="H27" s="10" t="s">
+        <v>367</v>
+      </c>
+      <c r="I27" s="11">
+        <v>-72729.899999999994</v>
+      </c>
+      <c r="J27" s="11">
+        <v>-78517.39</v>
+      </c>
+      <c r="K27" s="11">
+        <v>-67574.27</v>
+      </c>
+    </row>
+    <row r="28" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C28" s="12" t="s">
+        <v>368</v>
+      </c>
+      <c r="D28" s="13">
+        <v>-12904.36</v>
+      </c>
+      <c r="E28" s="13">
+        <v>-16703.75</v>
+      </c>
+      <c r="F28" s="13">
+        <v>-9258.25</v>
+      </c>
+      <c r="H28" s="12" t="s">
+        <v>368</v>
+      </c>
+      <c r="I28" s="13">
+        <v>-20678.3</v>
+      </c>
+      <c r="J28" s="13">
+        <v>-25853.46</v>
+      </c>
+      <c r="K28" s="13">
+        <v>-15745.36</v>
+      </c>
+    </row>
+    <row r="29" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C29" s="12" t="s">
+        <v>369</v>
+      </c>
+      <c r="D29" s="13">
+        <v>-7329.77</v>
+      </c>
+      <c r="E29" s="13">
+        <v>-10051.69</v>
+      </c>
+      <c r="F29" s="13">
+        <v>-4733.33</v>
+      </c>
+      <c r="H29" s="12" t="s">
+        <v>369</v>
+      </c>
+      <c r="I29" s="13">
+        <v>-15162.75</v>
+      </c>
+      <c r="J29" s="13">
+        <v>-18556.97</v>
+      </c>
+      <c r="K29" s="13">
+        <v>-12083.85</v>
+      </c>
+    </row>
+    <row r="30" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C30" s="12" t="s">
+        <v>370</v>
+      </c>
+      <c r="D30" s="13">
+        <v>-1755.18</v>
+      </c>
+      <c r="E30" s="13">
+        <v>-5679.75</v>
+      </c>
+      <c r="F30" s="13">
+        <v>2141.39</v>
+      </c>
+      <c r="H30" s="12" t="s">
+        <v>370</v>
+      </c>
+      <c r="I30" s="13">
+        <v>-9647.19</v>
+      </c>
+      <c r="J30" s="13">
+        <v>-11998.01</v>
+      </c>
+      <c r="K30" s="13">
+        <v>-7384.95</v>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="C2:F2"/>
+    <mergeCell ref="H2:K2"/>
+    <mergeCell ref="C18:F18"/>
+    <mergeCell ref="H18:K18"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D455D975-647C-424C-912C-DB92418F2207}">
+  <dimension ref="D4:N32"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="4" max="4" width="21.28515625" customWidth="1"/>
+    <col min="5" max="7" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="23.5703125" customWidth="1"/>
+    <col min="12" max="14" width="9.85546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="4" spans="4:14" x14ac:dyDescent="0.25">
+      <c r="D4" s="14" t="s">
+        <v>374</v>
+      </c>
+      <c r="E4" s="14"/>
+      <c r="F4" s="14"/>
+      <c r="G4" s="14"/>
+      <c r="K4" s="14" t="s">
+        <v>376</v>
+      </c>
+      <c r="L4" s="14"/>
+      <c r="M4" s="14"/>
+      <c r="N4" s="14"/>
+    </row>
+    <row r="5" spans="4:14" x14ac:dyDescent="0.25">
+      <c r="D5" s="15" t="s">
+        <v>356</v>
+      </c>
+      <c r="E5" s="16" t="s">
+        <v>371</v>
+      </c>
+      <c r="F5" s="16" t="s">
+        <v>372</v>
+      </c>
+      <c r="G5" s="16" t="s">
+        <v>373</v>
+      </c>
+      <c r="K5" s="8" t="s">
+        <v>356</v>
+      </c>
+      <c r="L5" s="9" t="s">
+        <v>371</v>
+      </c>
+      <c r="M5" s="9" t="s">
+        <v>372</v>
+      </c>
+      <c r="N5" s="9" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="6" spans="4:14" x14ac:dyDescent="0.25">
+      <c r="D6" s="17" t="s">
+        <v>360</v>
+      </c>
+      <c r="E6" s="18">
+        <v>-10398.52</v>
+      </c>
+      <c r="F6" s="18">
+        <v>-15013.72</v>
+      </c>
+      <c r="G6" s="18">
+        <v>-6014.7</v>
+      </c>
+      <c r="K6" s="21" t="s">
+        <v>360</v>
+      </c>
+      <c r="L6" s="22">
+        <v>-19663.169999999998</v>
+      </c>
+      <c r="M6" s="22">
+        <v>-27588.38</v>
+      </c>
+      <c r="N6" s="22">
+        <v>-12238.31</v>
+      </c>
+    </row>
+    <row r="7" spans="4:14" x14ac:dyDescent="0.25">
+      <c r="D7" s="17" t="s">
+        <v>361</v>
+      </c>
+      <c r="E7" s="18">
+        <v>2459.6999999999998</v>
+      </c>
+      <c r="F7" s="19">
+        <v>237.23</v>
+      </c>
+      <c r="G7" s="18">
+        <v>4792.01</v>
+      </c>
+      <c r="K7" s="21" t="s">
+        <v>361</v>
+      </c>
+      <c r="L7" s="22">
+        <v>5558.54</v>
+      </c>
+      <c r="M7" s="22">
+        <v>3135.62</v>
+      </c>
+      <c r="N7" s="22">
+        <v>8116.55</v>
+      </c>
+    </row>
+    <row r="8" spans="4:14" x14ac:dyDescent="0.25">
+      <c r="D8" s="17" t="s">
+        <v>362</v>
+      </c>
+      <c r="E8" s="18">
+        <v>5936.82</v>
+      </c>
+      <c r="F8" s="18">
+        <v>3595.79</v>
+      </c>
+      <c r="G8" s="18">
+        <v>8363.34</v>
+      </c>
+      <c r="K8" s="21" t="s">
+        <v>362</v>
+      </c>
+      <c r="L8" s="22">
+        <v>6666.07</v>
+      </c>
+      <c r="M8" s="22">
+        <v>4065.63</v>
+      </c>
+      <c r="N8" s="22">
+        <v>9435.7099999999991</v>
+      </c>
+    </row>
+    <row r="9" spans="4:14" x14ac:dyDescent="0.25">
+      <c r="D9" s="17" t="s">
+        <v>363</v>
+      </c>
+      <c r="E9" s="18">
+        <v>-2689.1</v>
+      </c>
+      <c r="F9" s="18">
+        <v>-3481.49</v>
+      </c>
+      <c r="G9" s="18">
+        <v>-2003.36</v>
+      </c>
+      <c r="K9" s="21" t="s">
+        <v>363</v>
+      </c>
+      <c r="L9" s="22">
+        <v>-3181.46</v>
+      </c>
+      <c r="M9" s="22">
+        <v>-4087.23</v>
+      </c>
+      <c r="N9" s="22">
+        <v>-2360.4699999999998</v>
+      </c>
+    </row>
+    <row r="10" spans="4:14" x14ac:dyDescent="0.25">
+      <c r="D10" s="17" t="s">
+        <v>364</v>
+      </c>
+      <c r="E10" s="19">
+        <v>-990.18</v>
+      </c>
+      <c r="F10" s="18">
+        <v>-1387.19</v>
+      </c>
+      <c r="G10" s="19">
+        <v>-623.53</v>
+      </c>
+      <c r="K10" s="21" t="s">
+        <v>364</v>
+      </c>
+      <c r="L10" s="22">
+        <v>-1730.97</v>
+      </c>
+      <c r="M10" s="22">
+        <v>-2233.73</v>
+      </c>
+      <c r="N10" s="22">
+        <v>-1278.6500000000001</v>
+      </c>
+    </row>
+    <row r="11" spans="4:14" x14ac:dyDescent="0.25">
+      <c r="D11" s="17" t="s">
+        <v>365</v>
+      </c>
+      <c r="E11" s="18">
+        <v>-9481.4500000000007</v>
+      </c>
+      <c r="F11" s="18">
+        <v>-12697.14</v>
+      </c>
+      <c r="G11" s="18">
+        <v>-6566.78</v>
+      </c>
+      <c r="K11" s="21" t="s">
+        <v>365</v>
+      </c>
+      <c r="L11" s="22">
+        <v>-7624.87</v>
+      </c>
+      <c r="M11" s="22">
+        <v>-10744.44</v>
+      </c>
+      <c r="N11" s="22">
+        <v>-4703.42</v>
+      </c>
+    </row>
+    <row r="12" spans="4:14" x14ac:dyDescent="0.25">
+      <c r="D12" s="17" t="s">
+        <v>366</v>
+      </c>
+      <c r="E12" s="18">
+        <v>-10000</v>
+      </c>
+      <c r="F12" s="18">
+        <v>-10000</v>
+      </c>
+      <c r="G12" s="18">
+        <v>-10000</v>
+      </c>
+      <c r="K12" s="21" t="s">
+        <v>366</v>
+      </c>
+      <c r="L12" s="22">
+        <v>-10000</v>
+      </c>
+      <c r="M12" s="22">
+        <v>-10000</v>
+      </c>
+      <c r="N12" s="22">
+        <v>-10000</v>
+      </c>
+    </row>
+    <row r="13" spans="4:14" x14ac:dyDescent="0.25">
+      <c r="D13" s="17" t="s">
+        <v>367</v>
+      </c>
+      <c r="E13" s="18">
+        <v>-59931.26</v>
+      </c>
+      <c r="F13" s="18">
+        <v>-67975.600000000006</v>
+      </c>
+      <c r="G13" s="18">
+        <v>-53204.22</v>
+      </c>
+      <c r="K13" s="21" t="s">
+        <v>367</v>
+      </c>
+      <c r="L13" s="22">
+        <v>-67057.27</v>
+      </c>
+      <c r="M13" s="22">
+        <v>-75177.960000000006</v>
+      </c>
+      <c r="N13" s="22">
+        <v>-59804.639999999999</v>
+      </c>
+    </row>
+    <row r="14" spans="4:14" x14ac:dyDescent="0.25">
+      <c r="D14" s="17" t="s">
+        <v>368</v>
+      </c>
+      <c r="E14" s="18">
+        <v>-4461.7</v>
+      </c>
+      <c r="F14" s="18">
+        <v>-7357.62</v>
+      </c>
+      <c r="G14" s="18">
+        <v>-1650.52</v>
+      </c>
+      <c r="K14" s="21" t="s">
+        <v>368</v>
+      </c>
+      <c r="L14" s="22">
+        <v>-12997.1</v>
+      </c>
+      <c r="M14" s="22">
+        <v>-18474.61</v>
+      </c>
+      <c r="N14" s="22">
+        <v>-7875.77</v>
+      </c>
+    </row>
+    <row r="15" spans="4:14" x14ac:dyDescent="0.25">
+      <c r="D15" s="17" t="s">
+        <v>369</v>
+      </c>
+      <c r="E15" s="18">
+        <v>1475.12</v>
+      </c>
+      <c r="F15" s="18">
+        <v>-1411.39</v>
+      </c>
+      <c r="G15" s="18">
+        <v>4280.53</v>
+      </c>
+      <c r="K15" s="21" t="s">
+        <v>369</v>
+      </c>
+      <c r="L15" s="22">
+        <v>-6331.03</v>
+      </c>
+      <c r="M15" s="22">
+        <v>-9858.7000000000007</v>
+      </c>
+      <c r="N15" s="22">
+        <v>-3073.31</v>
+      </c>
+    </row>
+    <row r="16" spans="4:14" x14ac:dyDescent="0.25">
+      <c r="D16" s="17" t="s">
+        <v>370</v>
+      </c>
+      <c r="E16" s="18">
+        <v>7411.93</v>
+      </c>
+      <c r="F16" s="18">
+        <v>3032.78</v>
+      </c>
+      <c r="G16" s="18">
+        <v>11922.09</v>
+      </c>
+      <c r="K16" s="21" t="s">
+        <v>370</v>
+      </c>
+      <c r="L16" s="21">
+        <v>335.04</v>
+      </c>
+      <c r="M16" s="22">
+        <v>-2757.19</v>
+      </c>
+      <c r="N16" s="22">
+        <v>3380.2</v>
+      </c>
+    </row>
+    <row r="20" spans="4:14" x14ac:dyDescent="0.25">
+      <c r="D20" s="14" t="s">
+        <v>375</v>
+      </c>
+      <c r="E20" s="14"/>
+      <c r="F20" s="14"/>
+      <c r="G20" s="14"/>
+      <c r="K20" s="14" t="s">
+        <v>377</v>
+      </c>
+      <c r="L20" s="14"/>
+      <c r="M20" s="14"/>
+      <c r="N20" s="14"/>
+    </row>
+    <row r="21" spans="4:14" x14ac:dyDescent="0.25">
+      <c r="D21" s="8" t="s">
+        <v>356</v>
+      </c>
+      <c r="E21" s="9" t="s">
+        <v>371</v>
+      </c>
+      <c r="F21" s="9" t="s">
+        <v>372</v>
+      </c>
+      <c r="G21" s="9" t="s">
+        <v>373</v>
+      </c>
+      <c r="K21" s="8" t="s">
+        <v>356</v>
+      </c>
+      <c r="L21" s="9" t="s">
+        <v>371</v>
+      </c>
+      <c r="M21" s="9" t="s">
+        <v>372</v>
+      </c>
+      <c r="N21" s="9" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="22" spans="4:14" x14ac:dyDescent="0.25">
+      <c r="D22" s="10" t="s">
+        <v>360</v>
+      </c>
+      <c r="E22" s="20">
+        <v>-21843.040000000001</v>
+      </c>
+      <c r="F22" s="20">
+        <v>-26025.27</v>
+      </c>
+      <c r="G22" s="20">
+        <v>-18077.8</v>
+      </c>
+      <c r="K22" s="10" t="s">
+        <v>360</v>
+      </c>
+      <c r="L22" s="20">
+        <v>-37292.04</v>
+      </c>
+      <c r="M22" s="20">
+        <v>-44691.58</v>
+      </c>
+      <c r="N22" s="20">
+        <v>-30212.42</v>
+      </c>
+    </row>
+    <row r="23" spans="4:14" x14ac:dyDescent="0.25">
+      <c r="D23" s="10" t="s">
+        <v>361</v>
+      </c>
+      <c r="E23" s="20">
+        <v>-3871.75</v>
+      </c>
+      <c r="F23" s="20">
+        <v>-5465.71</v>
+      </c>
+      <c r="G23" s="20">
+        <v>-2349.6999999999998</v>
+      </c>
+      <c r="K23" s="10" t="s">
+        <v>361</v>
+      </c>
+      <c r="L23" s="20">
+        <v>-2553.63</v>
+      </c>
+      <c r="M23" s="20">
+        <v>-4293.0200000000004</v>
+      </c>
+      <c r="N23" s="11">
+        <v>-866.01</v>
+      </c>
+    </row>
+    <row r="24" spans="4:14" x14ac:dyDescent="0.25">
+      <c r="D24" s="10" t="s">
+        <v>362</v>
+      </c>
+      <c r="E24" s="20">
+        <v>2911.47</v>
+      </c>
+      <c r="F24" s="11">
+        <v>790.28</v>
+      </c>
+      <c r="G24" s="20">
+        <v>5033.82</v>
+      </c>
+      <c r="K24" s="10" t="s">
+        <v>362</v>
+      </c>
+      <c r="L24" s="20">
+        <v>6879.6</v>
+      </c>
+      <c r="M24" s="20">
+        <v>4530.62</v>
+      </c>
+      <c r="N24" s="20">
+        <v>9341.39</v>
+      </c>
+    </row>
+    <row r="25" spans="4:14" x14ac:dyDescent="0.25">
+      <c r="D25" s="10" t="s">
+        <v>363</v>
+      </c>
+      <c r="E25" s="20">
+        <v>-1807.76</v>
+      </c>
+      <c r="F25" s="20">
+        <v>-2297.3000000000002</v>
+      </c>
+      <c r="G25" s="20">
+        <v>-1355.81</v>
+      </c>
+      <c r="K25" s="10" t="s">
+        <v>363</v>
+      </c>
+      <c r="L25" s="20">
+        <v>-3495.43</v>
+      </c>
+      <c r="M25" s="20">
+        <v>-4185.75</v>
+      </c>
+      <c r="N25" s="20">
+        <v>-2852.75</v>
+      </c>
+    </row>
+    <row r="26" spans="4:14" x14ac:dyDescent="0.25">
+      <c r="D26" s="10" t="s">
+        <v>364</v>
+      </c>
+      <c r="E26" s="11">
+        <v>-748.36</v>
+      </c>
+      <c r="F26" s="20">
+        <v>-1013.94</v>
+      </c>
+      <c r="G26" s="11">
+        <v>-495.16</v>
+      </c>
+      <c r="K26" s="10" t="s">
+        <v>364</v>
+      </c>
+      <c r="L26" s="20">
+        <v>-1563.79</v>
+      </c>
+      <c r="M26" s="20">
+        <v>-1934.13</v>
+      </c>
+      <c r="N26" s="20">
+        <v>-1206.94</v>
+      </c>
+    </row>
+    <row r="27" spans="4:14" x14ac:dyDescent="0.25">
+      <c r="D27" s="10" t="s">
+        <v>365</v>
+      </c>
+      <c r="E27" s="20">
+        <v>-7843.18</v>
+      </c>
+      <c r="F27" s="20">
+        <v>-9933.56</v>
+      </c>
+      <c r="G27" s="20">
+        <v>-5906.78</v>
+      </c>
+      <c r="K27" s="10" t="s">
+        <v>365</v>
+      </c>
+      <c r="L27" s="20">
+        <v>-8362.82</v>
+      </c>
+      <c r="M27" s="20">
+        <v>-10744.62</v>
+      </c>
+      <c r="N27" s="20">
+        <v>-6158.73</v>
+      </c>
+    </row>
+    <row r="28" spans="4:14" x14ac:dyDescent="0.25">
+      <c r="D28" s="10" t="s">
+        <v>366</v>
+      </c>
+      <c r="E28" s="20">
+        <v>-10000</v>
+      </c>
+      <c r="F28" s="20">
+        <v>-10000</v>
+      </c>
+      <c r="G28" s="20">
+        <v>-10000</v>
+      </c>
+      <c r="K28" s="10" t="s">
+        <v>366</v>
+      </c>
+      <c r="L28" s="20">
+        <v>-10000</v>
+      </c>
+      <c r="M28" s="20">
+        <v>-10000</v>
+      </c>
+      <c r="N28" s="20">
+        <v>-10000</v>
+      </c>
+    </row>
+    <row r="29" spans="4:14" x14ac:dyDescent="0.25">
+      <c r="D29" s="10" t="s">
+        <v>367</v>
+      </c>
+      <c r="E29" s="20">
+        <v>-52707.519999999997</v>
+      </c>
+      <c r="F29" s="20">
+        <v>-57739.01</v>
+      </c>
+      <c r="G29" s="20">
+        <v>-48325.32</v>
+      </c>
+      <c r="K29" s="10" t="s">
+        <v>367</v>
+      </c>
+      <c r="L29" s="20">
+        <v>-70028.12</v>
+      </c>
+      <c r="M29" s="20">
+        <v>-76379.990000000005</v>
+      </c>
+      <c r="N29" s="20">
+        <v>-64268.62</v>
+      </c>
+    </row>
+    <row r="30" spans="4:14" x14ac:dyDescent="0.25">
+      <c r="D30" s="10" t="s">
+        <v>368</v>
+      </c>
+      <c r="E30" s="20">
+        <v>-18931.57</v>
+      </c>
+      <c r="F30" s="20">
+        <v>-21858.91</v>
+      </c>
+      <c r="G30" s="20">
+        <v>-16311.9</v>
+      </c>
+      <c r="K30" s="10" t="s">
+        <v>368</v>
+      </c>
+      <c r="L30" s="20">
+        <v>-30412.44</v>
+      </c>
+      <c r="M30" s="20">
+        <v>-35761.49</v>
+      </c>
+      <c r="N30" s="20">
+        <v>-25444.03</v>
+      </c>
+    </row>
+    <row r="31" spans="4:14" x14ac:dyDescent="0.25">
+      <c r="D31" s="10" t="s">
+        <v>369</v>
+      </c>
+      <c r="E31" s="20">
+        <v>-16020.11</v>
+      </c>
+      <c r="F31" s="20">
+        <v>-19065.13</v>
+      </c>
+      <c r="G31" s="20">
+        <v>-13262.47</v>
+      </c>
+      <c r="K31" s="10" t="s">
+        <v>369</v>
+      </c>
+      <c r="L31" s="20">
+        <v>-23532.83</v>
+      </c>
+      <c r="M31" s="20">
+        <v>-27192.51</v>
+      </c>
+      <c r="N31" s="20">
+        <v>-20213.02</v>
+      </c>
+    </row>
+    <row r="32" spans="4:14" x14ac:dyDescent="0.25">
+      <c r="D32" s="10" t="s">
+        <v>370</v>
+      </c>
+      <c r="E32" s="20">
+        <v>-13108.64</v>
+      </c>
+      <c r="F32" s="20">
+        <v>-17543.400000000001</v>
+      </c>
+      <c r="G32" s="20">
+        <v>-8937.5499999999993</v>
+      </c>
+      <c r="K32" s="10" t="s">
+        <v>370</v>
+      </c>
+      <c r="L32" s="20">
+        <v>-16653.23</v>
+      </c>
+      <c r="M32" s="20">
+        <v>-19897.689999999999</v>
+      </c>
+      <c r="N32" s="20">
+        <v>-13666.57</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="D4:G4"/>
+    <mergeCell ref="D20:G20"/>
+    <mergeCell ref="K4:N4"/>
+    <mergeCell ref="K20:N20"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B037BF0F-D82F-44E6-8F07-AC277E10E42D}">
   <dimension ref="B2:F73"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2357,10 +3569,10 @@
   <sheetData>
     <row r="2" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B2" s="3" t="s">
-        <v>121</v>
+        <v>43</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>122</v>
+        <v>44</v>
       </c>
     </row>
     <row r="3" spans="2:6" x14ac:dyDescent="0.25">
@@ -2381,74 +3593,74 @@
     </row>
     <row r="5" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B5" s="1" t="s">
-        <v>107</v>
+        <v>29</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>123</v>
+        <v>45</v>
       </c>
     </row>
     <row r="6" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B6" s="1" t="s">
-        <v>108</v>
+        <v>30</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>124</v>
+        <v>46</v>
       </c>
     </row>
     <row r="7" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B7" s="1" t="s">
-        <v>109</v>
+        <v>31</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>125</v>
+        <v>47</v>
       </c>
     </row>
     <row r="8" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B8" s="1" t="s">
-        <v>110</v>
+        <v>32</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>126</v>
+        <v>48</v>
       </c>
     </row>
     <row r="9" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B9" s="1" t="s">
-        <v>111</v>
+        <v>33</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>127</v>
+        <v>49</v>
       </c>
     </row>
     <row r="10" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B10" s="1" t="s">
-        <v>112</v>
+        <v>34</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>128</v>
+        <v>50</v>
       </c>
     </row>
     <row r="11" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B11" s="1" t="s">
-        <v>113</v>
+        <v>35</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>129</v>
+        <v>51</v>
       </c>
     </row>
     <row r="12" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B12" s="1" t="s">
-        <v>114</v>
+        <v>36</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>130</v>
+        <v>52</v>
       </c>
     </row>
     <row r="13" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B13" s="1" t="s">
-        <v>115</v>
+        <v>37</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>131</v>
+        <v>53</v>
       </c>
     </row>
     <row r="14" spans="2:6" x14ac:dyDescent="0.25">
@@ -2477,66 +3689,66 @@
     </row>
     <row r="17" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B17" s="1" t="s">
-        <v>116</v>
+        <v>38</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>132</v>
+        <v>54</v>
       </c>
     </row>
     <row r="18" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B18" s="1" t="s">
-        <v>83</v>
+        <v>22</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>101</v>
+        <v>27</v>
       </c>
     </row>
     <row r="19" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B19" s="1" t="s">
-        <v>117</v>
+        <v>39</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>133</v>
+        <v>55</v>
       </c>
     </row>
     <row r="20" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B20" s="1" t="s">
-        <v>118</v>
+        <v>40</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>134</v>
+        <v>56</v>
       </c>
     </row>
     <row r="21" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B21" s="1" t="s">
-        <v>119</v>
+        <v>41</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>135</v>
+        <v>57</v>
       </c>
     </row>
     <row r="22" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B22" s="1" t="s">
-        <v>120</v>
+        <v>42</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>136</v>
+        <v>58</v>
       </c>
     </row>
     <row r="23" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B23" s="2" t="s">
-        <v>88</v>
+        <v>23</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>106</v>
+        <v>28</v>
       </c>
     </row>
     <row r="27" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B27" s="3" t="s">
-        <v>151</v>
+        <v>73</v>
       </c>
       <c r="F27" s="3" t="s">
-        <v>167</v>
+        <v>89</v>
       </c>
     </row>
     <row r="28" spans="2:6" x14ac:dyDescent="0.25">
@@ -2552,79 +3764,79 @@
         <v>13</v>
       </c>
       <c r="F29" s="1" t="s">
-        <v>152</v>
+        <v>74</v>
       </c>
     </row>
     <row r="30" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B30" s="1" t="s">
-        <v>137</v>
+        <v>59</v>
       </c>
       <c r="F30" s="1" t="s">
-        <v>153</v>
+        <v>75</v>
       </c>
     </row>
     <row r="31" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B31" s="1" t="s">
-        <v>138</v>
+        <v>60</v>
       </c>
       <c r="F31" s="1" t="s">
-        <v>154</v>
+        <v>76</v>
       </c>
     </row>
     <row r="32" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B32" s="1" t="s">
-        <v>139</v>
+        <v>61</v>
       </c>
       <c r="F32" s="1" t="s">
-        <v>155</v>
+        <v>77</v>
       </c>
     </row>
     <row r="33" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B33" s="1" t="s">
-        <v>140</v>
+        <v>62</v>
       </c>
       <c r="F33" s="1" t="s">
-        <v>156</v>
+        <v>78</v>
       </c>
     </row>
     <row r="34" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B34" s="1" t="s">
-        <v>141</v>
+        <v>63</v>
       </c>
       <c r="F34" s="1" t="s">
-        <v>157</v>
+        <v>79</v>
       </c>
     </row>
     <row r="35" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B35" s="1" t="s">
-        <v>142</v>
+        <v>64</v>
       </c>
       <c r="F35" s="1" t="s">
-        <v>158</v>
+        <v>80</v>
       </c>
     </row>
     <row r="36" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B36" s="1" t="s">
-        <v>143</v>
+        <v>65</v>
       </c>
       <c r="F36" s="1" t="s">
-        <v>159</v>
+        <v>81</v>
       </c>
     </row>
     <row r="37" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B37" s="1" t="s">
-        <v>144</v>
+        <v>66</v>
       </c>
       <c r="F37" s="1" t="s">
-        <v>160</v>
+        <v>82</v>
       </c>
     </row>
     <row r="38" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B38" s="1" t="s">
-        <v>145</v>
+        <v>67</v>
       </c>
       <c r="F38" s="1" t="s">
-        <v>161</v>
+        <v>83</v>
       </c>
     </row>
     <row r="39" spans="2:6" x14ac:dyDescent="0.25">
@@ -2653,66 +3865,66 @@
     </row>
     <row r="42" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B42" s="1" t="s">
-        <v>146</v>
+        <v>68</v>
       </c>
       <c r="F42" s="1" t="s">
-        <v>162</v>
+        <v>84</v>
       </c>
     </row>
     <row r="43" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B43" s="1" t="s">
-        <v>83</v>
+        <v>22</v>
       </c>
       <c r="F43" s="1" t="s">
-        <v>101</v>
+        <v>27</v>
       </c>
     </row>
     <row r="44" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B44" s="1" t="s">
-        <v>147</v>
+        <v>69</v>
       </c>
       <c r="F44" s="1" t="s">
-        <v>163</v>
+        <v>85</v>
       </c>
     </row>
     <row r="45" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B45" s="1" t="s">
-        <v>148</v>
+        <v>70</v>
       </c>
       <c r="F45" s="1" t="s">
-        <v>164</v>
+        <v>86</v>
       </c>
     </row>
     <row r="46" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B46" s="1" t="s">
-        <v>149</v>
+        <v>71</v>
       </c>
       <c r="F46" s="1" t="s">
-        <v>165</v>
+        <v>87</v>
       </c>
     </row>
     <row r="47" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B47" s="1" t="s">
-        <v>150</v>
+        <v>72</v>
       </c>
       <c r="F47" s="1" t="s">
-        <v>166</v>
+        <v>88</v>
       </c>
     </row>
     <row r="48" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B48" s="2" t="s">
-        <v>88</v>
+        <v>23</v>
       </c>
       <c r="F48" s="2" t="s">
-        <v>106</v>
+        <v>28</v>
       </c>
     </row>
     <row r="52" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B52" s="3" t="s">
-        <v>197</v>
+        <v>119</v>
       </c>
       <c r="F52" s="3" t="s">
-        <v>196</v>
+        <v>118</v>
       </c>
     </row>
     <row r="53" spans="2:6" x14ac:dyDescent="0.25">
@@ -2733,74 +3945,74 @@
     </row>
     <row r="55" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B55" s="1" t="s">
-        <v>168</v>
+        <v>90</v>
       </c>
       <c r="F55" s="1" t="s">
-        <v>182</v>
+        <v>104</v>
       </c>
     </row>
     <row r="56" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B56" s="1" t="s">
-        <v>169</v>
+        <v>91</v>
       </c>
       <c r="F56" s="1" t="s">
-        <v>183</v>
+        <v>105</v>
       </c>
     </row>
     <row r="57" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B57" s="1" t="s">
-        <v>170</v>
+        <v>92</v>
       </c>
       <c r="F57" s="1" t="s">
-        <v>184</v>
+        <v>106</v>
       </c>
     </row>
     <row r="58" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B58" s="1" t="s">
-        <v>171</v>
+        <v>93</v>
       </c>
       <c r="F58" s="1" t="s">
-        <v>185</v>
+        <v>107</v>
       </c>
     </row>
     <row r="59" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B59" s="1" t="s">
-        <v>172</v>
+        <v>94</v>
       </c>
       <c r="F59" s="1" t="s">
-        <v>186</v>
+        <v>108</v>
       </c>
     </row>
     <row r="60" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B60" s="1" t="s">
-        <v>173</v>
+        <v>95</v>
       </c>
       <c r="F60" s="1" t="s">
-        <v>187</v>
+        <v>109</v>
       </c>
     </row>
     <row r="61" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B61" s="1" t="s">
-        <v>174</v>
+        <v>96</v>
       </c>
       <c r="F61" s="1" t="s">
-        <v>188</v>
+        <v>110</v>
       </c>
     </row>
     <row r="62" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B62" s="1" t="s">
-        <v>175</v>
+        <v>97</v>
       </c>
       <c r="F62" s="1" t="s">
-        <v>189</v>
+        <v>111</v>
       </c>
     </row>
     <row r="63" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B63" s="1" t="s">
-        <v>176</v>
+        <v>98</v>
       </c>
       <c r="F63" s="1" t="s">
-        <v>190</v>
+        <v>112</v>
       </c>
     </row>
     <row r="64" spans="2:6" x14ac:dyDescent="0.25">
@@ -2829,58 +4041,58 @@
     </row>
     <row r="67" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B67" s="1" t="s">
-        <v>177</v>
+        <v>99</v>
       </c>
       <c r="F67" s="1" t="s">
-        <v>191</v>
+        <v>113</v>
       </c>
     </row>
     <row r="68" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B68" s="1" t="s">
-        <v>83</v>
+        <v>22</v>
       </c>
       <c r="F68" s="1" t="s">
-        <v>101</v>
+        <v>27</v>
       </c>
     </row>
     <row r="69" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B69" s="1" t="s">
-        <v>178</v>
+        <v>100</v>
       </c>
       <c r="F69" s="1" t="s">
-        <v>192</v>
+        <v>114</v>
       </c>
     </row>
     <row r="70" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B70" s="1" t="s">
-        <v>179</v>
+        <v>101</v>
       </c>
       <c r="F70" s="1" t="s">
-        <v>193</v>
+        <v>115</v>
       </c>
     </row>
     <row r="71" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B71" s="1" t="s">
-        <v>180</v>
+        <v>102</v>
       </c>
       <c r="F71" s="1" t="s">
-        <v>194</v>
+        <v>116</v>
       </c>
     </row>
     <row r="72" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B72" s="1" t="s">
-        <v>181</v>
+        <v>103</v>
       </c>
       <c r="F72" s="1" t="s">
-        <v>195</v>
+        <v>117</v>
       </c>
     </row>
     <row r="73" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B73" s="2" t="s">
-        <v>88</v>
+        <v>23</v>
       </c>
       <c r="F73" s="2" t="s">
-        <v>106</v>
+        <v>28</v>
       </c>
     </row>
   </sheetData>
@@ -2888,7 +4100,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6055C001-9D9E-41A1-8DE6-C0D19D2977B2}">
   <dimension ref="B2:G40"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2899,266 +4111,266 @@
   <sheetData>
     <row r="2" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B2" s="3" t="s">
-        <v>332</v>
+        <v>214</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>343</v>
+        <v>225</v>
       </c>
     </row>
     <row r="3" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3" s="1" t="s">
-        <v>282</v>
+        <v>204</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>333</v>
+        <v>215</v>
       </c>
     </row>
     <row r="4" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B4" s="1" t="s">
-        <v>324</v>
+        <v>206</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>334</v>
+        <v>216</v>
       </c>
     </row>
     <row r="5" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B5" s="1" t="s">
-        <v>325</v>
+        <v>207</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>335</v>
+        <v>217</v>
       </c>
     </row>
     <row r="6" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B6" s="1" t="s">
-        <v>326</v>
+        <v>208</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>336</v>
+        <v>218</v>
       </c>
     </row>
     <row r="7" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B7" s="1" t="s">
-        <v>327</v>
+        <v>209</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>337</v>
+        <v>219</v>
       </c>
     </row>
     <row r="8" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B8" s="1" t="s">
-        <v>328</v>
+        <v>210</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>338</v>
+        <v>220</v>
       </c>
     </row>
     <row r="9" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B9" s="1" t="s">
-        <v>329</v>
+        <v>211</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>339</v>
+        <v>221</v>
       </c>
     </row>
     <row r="10" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B10" s="1" t="s">
-        <v>289</v>
+        <v>205</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>340</v>
+        <v>222</v>
       </c>
     </row>
     <row r="11" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B11" s="1" t="s">
-        <v>330</v>
+        <v>212</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>341</v>
+        <v>223</v>
       </c>
     </row>
     <row r="12" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B12" s="2" t="s">
-        <v>331</v>
+        <v>213</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>342</v>
+        <v>224</v>
       </c>
     </row>
     <row r="16" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B16" s="3" t="s">
-        <v>354</v>
+        <v>236</v>
       </c>
       <c r="G16" s="3" t="s">
-        <v>363</v>
+        <v>245</v>
       </c>
     </row>
     <row r="17" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B17" s="1" t="s">
-        <v>344</v>
+        <v>226</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>344</v>
+        <v>226</v>
       </c>
     </row>
     <row r="18" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B18" s="1" t="s">
-        <v>345</v>
+        <v>227</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>355</v>
+        <v>237</v>
       </c>
     </row>
     <row r="19" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B19" s="1" t="s">
-        <v>346</v>
+        <v>228</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>356</v>
+        <v>238</v>
       </c>
     </row>
     <row r="20" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B20" s="1" t="s">
-        <v>347</v>
+        <v>229</v>
       </c>
       <c r="G20" s="1" t="s">
-        <v>357</v>
+        <v>239</v>
       </c>
     </row>
     <row r="21" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B21" s="1" t="s">
-        <v>348</v>
+        <v>230</v>
       </c>
       <c r="G21" s="1" t="s">
-        <v>358</v>
+        <v>240</v>
       </c>
     </row>
     <row r="22" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B22" s="1" t="s">
-        <v>349</v>
+        <v>231</v>
       </c>
       <c r="G22" s="1" t="s">
-        <v>359</v>
+        <v>241</v>
       </c>
     </row>
     <row r="23" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B23" s="1" t="s">
-        <v>350</v>
+        <v>232</v>
       </c>
       <c r="G23" s="1" t="s">
-        <v>360</v>
+        <v>242</v>
       </c>
     </row>
     <row r="24" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B24" s="1" t="s">
-        <v>351</v>
+        <v>233</v>
       </c>
       <c r="G24" s="1" t="s">
-        <v>351</v>
+        <v>233</v>
       </c>
     </row>
     <row r="25" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B25" s="1" t="s">
-        <v>352</v>
+        <v>234</v>
       </c>
       <c r="G25" s="1" t="s">
-        <v>361</v>
+        <v>243</v>
       </c>
     </row>
     <row r="26" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B26" s="2" t="s">
-        <v>353</v>
+        <v>235</v>
       </c>
       <c r="G26" s="2" t="s">
-        <v>362</v>
+        <v>244</v>
       </c>
     </row>
     <row r="30" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B30" s="3" t="s">
-        <v>372</v>
+        <v>254</v>
       </c>
       <c r="G30" s="3" t="s">
-        <v>381</v>
+        <v>263</v>
       </c>
     </row>
     <row r="31" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B31" s="1" t="s">
-        <v>282</v>
+        <v>204</v>
       </c>
       <c r="G31" s="1" t="s">
-        <v>333</v>
+        <v>215</v>
       </c>
     </row>
     <row r="32" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B32" s="1" t="s">
-        <v>364</v>
+        <v>246</v>
       </c>
       <c r="G32" s="1" t="s">
-        <v>373</v>
+        <v>255</v>
       </c>
     </row>
     <row r="33" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B33" s="1" t="s">
-        <v>365</v>
+        <v>247</v>
       </c>
       <c r="G33" s="1" t="s">
-        <v>374</v>
+        <v>256</v>
       </c>
     </row>
     <row r="34" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B34" s="1" t="s">
-        <v>366</v>
+        <v>248</v>
       </c>
       <c r="G34" s="1" t="s">
-        <v>375</v>
+        <v>257</v>
       </c>
     </row>
     <row r="35" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B35" s="1" t="s">
-        <v>367</v>
+        <v>249</v>
       </c>
       <c r="G35" s="1" t="s">
-        <v>376</v>
+        <v>258</v>
       </c>
     </row>
     <row r="36" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B36" s="1" t="s">
-        <v>368</v>
+        <v>250</v>
       </c>
       <c r="G36" s="1" t="s">
-        <v>377</v>
+        <v>259</v>
       </c>
     </row>
     <row r="37" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B37" s="1" t="s">
-        <v>369</v>
+        <v>251</v>
       </c>
       <c r="G37" s="1" t="s">
-        <v>378</v>
+        <v>260</v>
       </c>
     </row>
     <row r="38" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B38" s="1" t="s">
-        <v>289</v>
+        <v>205</v>
       </c>
       <c r="G38" s="1" t="s">
-        <v>340</v>
+        <v>222</v>
       </c>
     </row>
     <row r="39" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B39" s="1" t="s">
-        <v>370</v>
+        <v>252</v>
       </c>
       <c r="G39" s="1" t="s">
-        <v>379</v>
+        <v>261</v>
       </c>
     </row>
     <row r="40" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B40" s="2" t="s">
-        <v>371</v>
+        <v>253</v>
       </c>
       <c r="G40" s="2" t="s">
-        <v>380</v>
+        <v>262</v>
       </c>
     </row>
   </sheetData>
@@ -3166,7 +4378,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6F66DE85-36DD-44E9-82B9-5B77DC8C376F}">
   <dimension ref="B2:F70"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3177,10 +4389,10 @@
   <sheetData>
     <row r="2" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B2" s="3" t="s">
-        <v>211</v>
+        <v>133</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>225</v>
+        <v>147</v>
       </c>
     </row>
     <row r="3" spans="2:6" x14ac:dyDescent="0.25">
@@ -3196,71 +4408,71 @@
         <v>1</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>91</v>
+        <v>26</v>
       </c>
     </row>
     <row r="5" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B5" s="1" t="s">
-        <v>198</v>
+        <v>120</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>212</v>
+        <v>134</v>
       </c>
     </row>
     <row r="6" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B6" s="1" t="s">
-        <v>199</v>
+        <v>121</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>213</v>
+        <v>135</v>
       </c>
     </row>
     <row r="7" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B7" s="1" t="s">
-        <v>200</v>
+        <v>122</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>214</v>
+        <v>136</v>
       </c>
     </row>
     <row r="8" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B8" s="1" t="s">
-        <v>201</v>
+        <v>123</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>215</v>
+        <v>137</v>
       </c>
     </row>
     <row r="9" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B9" s="1" t="s">
-        <v>202</v>
+        <v>124</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>216</v>
+        <v>138</v>
       </c>
     </row>
     <row r="10" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B10" s="1" t="s">
-        <v>203</v>
+        <v>125</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>217</v>
+        <v>139</v>
       </c>
     </row>
     <row r="11" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B11" s="1" t="s">
-        <v>204</v>
+        <v>126</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>218</v>
+        <v>140</v>
       </c>
     </row>
     <row r="12" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B12" s="1" t="s">
-        <v>205</v>
+        <v>127</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>219</v>
+        <v>141</v>
       </c>
     </row>
     <row r="13" spans="2:6" x14ac:dyDescent="0.25">
@@ -3289,66 +4501,66 @@
     </row>
     <row r="16" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B16" s="1" t="s">
-        <v>206</v>
+        <v>128</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>220</v>
+        <v>142</v>
       </c>
     </row>
     <row r="17" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B17" s="1" t="s">
-        <v>83</v>
+        <v>22</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>101</v>
+        <v>27</v>
       </c>
     </row>
     <row r="18" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B18" s="1" t="s">
-        <v>207</v>
+        <v>129</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>221</v>
+        <v>143</v>
       </c>
     </row>
     <row r="19" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B19" s="1" t="s">
-        <v>208</v>
+        <v>130</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>222</v>
+        <v>144</v>
       </c>
     </row>
     <row r="20" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B20" s="1" t="s">
-        <v>209</v>
+        <v>131</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>223</v>
+        <v>145</v>
       </c>
     </row>
     <row r="21" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B21" s="1" t="s">
-        <v>210</v>
+        <v>132</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>224</v>
+        <v>146</v>
       </c>
     </row>
     <row r="22" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B22" s="2" t="s">
-        <v>88</v>
+        <v>23</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>106</v>
+        <v>28</v>
       </c>
     </row>
     <row r="25" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B25" s="3" t="s">
-        <v>239</v>
+        <v>161</v>
       </c>
       <c r="F25" s="3" t="s">
-        <v>253</v>
+        <v>175</v>
       </c>
     </row>
     <row r="26" spans="2:6" x14ac:dyDescent="0.25">
@@ -3369,66 +4581,66 @@
     </row>
     <row r="28" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B28" s="1" t="s">
-        <v>226</v>
+        <v>148</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>240</v>
+        <v>162</v>
       </c>
     </row>
     <row r="29" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B29" s="1" t="s">
-        <v>227</v>
+        <v>149</v>
       </c>
       <c r="F29" s="1" t="s">
-        <v>241</v>
+        <v>163</v>
       </c>
     </row>
     <row r="30" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B30" s="1" t="s">
-        <v>228</v>
+        <v>150</v>
       </c>
       <c r="F30" s="1" t="s">
-        <v>242</v>
+        <v>164</v>
       </c>
     </row>
     <row r="31" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B31" s="1" t="s">
-        <v>229</v>
+        <v>151</v>
       </c>
       <c r="F31" s="1" t="s">
-        <v>243</v>
+        <v>165</v>
       </c>
     </row>
     <row r="32" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B32" s="1" t="s">
-        <v>230</v>
+        <v>152</v>
       </c>
       <c r="F32" s="1" t="s">
-        <v>244</v>
+        <v>166</v>
       </c>
     </row>
     <row r="33" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B33" s="1" t="s">
-        <v>231</v>
+        <v>153</v>
       </c>
       <c r="F33" s="1" t="s">
-        <v>245</v>
+        <v>167</v>
       </c>
     </row>
     <row r="34" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B34" s="1" t="s">
-        <v>232</v>
+        <v>154</v>
       </c>
       <c r="F34" s="1" t="s">
-        <v>246</v>
+        <v>168</v>
       </c>
     </row>
     <row r="35" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B35" s="1" t="s">
-        <v>233</v>
+        <v>155</v>
       </c>
       <c r="F35" s="1" t="s">
-        <v>247</v>
+        <v>169</v>
       </c>
     </row>
     <row r="36" spans="2:6" x14ac:dyDescent="0.25">
@@ -3457,66 +4669,66 @@
     </row>
     <row r="39" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B39" s="1" t="s">
-        <v>234</v>
+        <v>156</v>
       </c>
       <c r="F39" s="1" t="s">
-        <v>248</v>
+        <v>170</v>
       </c>
     </row>
     <row r="40" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B40" s="1" t="s">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="F40" s="1" t="s">
-        <v>53</v>
+        <v>18</v>
       </c>
     </row>
     <row r="41" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B41" s="1" t="s">
-        <v>235</v>
+        <v>157</v>
       </c>
       <c r="F41" s="1" t="s">
-        <v>249</v>
+        <v>171</v>
       </c>
     </row>
     <row r="42" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B42" s="1" t="s">
-        <v>236</v>
+        <v>158</v>
       </c>
       <c r="F42" s="1" t="s">
-        <v>250</v>
+        <v>172</v>
       </c>
     </row>
     <row r="43" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B43" s="1" t="s">
-        <v>237</v>
+        <v>159</v>
       </c>
       <c r="F43" s="1" t="s">
-        <v>251</v>
+        <v>173</v>
       </c>
     </row>
     <row r="44" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B44" s="1" t="s">
-        <v>238</v>
+        <v>160</v>
       </c>
       <c r="F44" s="1" t="s">
-        <v>252</v>
+        <v>174</v>
       </c>
     </row>
     <row r="45" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B45" s="2" t="s">
-        <v>28</v>
+        <v>15</v>
       </c>
       <c r="F45" s="2" t="s">
-        <v>58</v>
+        <v>19</v>
       </c>
     </row>
     <row r="49" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B49" s="3" t="s">
-        <v>267</v>
+        <v>189</v>
       </c>
       <c r="F49" s="3" t="s">
-        <v>281</v>
+        <v>203</v>
       </c>
     </row>
     <row r="51" spans="2:6" x14ac:dyDescent="0.25">
@@ -3537,66 +4749,66 @@
     </row>
     <row r="53" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B53" s="1" t="s">
-        <v>254</v>
+        <v>176</v>
       </c>
       <c r="F53" s="1" t="s">
-        <v>268</v>
+        <v>190</v>
       </c>
     </row>
     <row r="54" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B54" s="1" t="s">
-        <v>255</v>
+        <v>177</v>
       </c>
       <c r="F54" s="1" t="s">
-        <v>269</v>
+        <v>191</v>
       </c>
     </row>
     <row r="55" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B55" s="1" t="s">
-        <v>256</v>
+        <v>178</v>
       </c>
       <c r="F55" s="1" t="s">
-        <v>270</v>
+        <v>192</v>
       </c>
     </row>
     <row r="56" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B56" s="1" t="s">
-        <v>257</v>
+        <v>179</v>
       </c>
       <c r="F56" s="1" t="s">
-        <v>271</v>
+        <v>193</v>
       </c>
     </row>
     <row r="57" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B57" s="1" t="s">
-        <v>258</v>
+        <v>180</v>
       </c>
       <c r="F57" s="1" t="s">
-        <v>272</v>
+        <v>194</v>
       </c>
     </row>
     <row r="58" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B58" s="1" t="s">
-        <v>259</v>
+        <v>181</v>
       </c>
       <c r="F58" s="1" t="s">
-        <v>273</v>
+        <v>195</v>
       </c>
     </row>
     <row r="59" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B59" s="1" t="s">
-        <v>260</v>
+        <v>182</v>
       </c>
       <c r="F59" s="1" t="s">
-        <v>274</v>
+        <v>196</v>
       </c>
     </row>
     <row r="60" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B60" s="1" t="s">
-        <v>261</v>
+        <v>183</v>
       </c>
       <c r="F60" s="1" t="s">
-        <v>275</v>
+        <v>197</v>
       </c>
     </row>
     <row r="61" spans="2:6" x14ac:dyDescent="0.25">
@@ -3625,58 +4837,58 @@
     </row>
     <row r="64" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B64" s="1" t="s">
-        <v>262</v>
+        <v>184</v>
       </c>
       <c r="F64" s="1" t="s">
-        <v>276</v>
+        <v>198</v>
       </c>
     </row>
     <row r="65" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B65" s="1" t="s">
-        <v>38</v>
+        <v>16</v>
       </c>
       <c r="F65" s="1" t="s">
-        <v>68</v>
+        <v>20</v>
       </c>
     </row>
     <row r="66" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B66" s="1" t="s">
-        <v>263</v>
+        <v>185</v>
       </c>
       <c r="F66" s="1" t="s">
-        <v>277</v>
+        <v>199</v>
       </c>
     </row>
     <row r="67" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B67" s="1" t="s">
-        <v>264</v>
+        <v>186</v>
       </c>
       <c r="F67" s="1" t="s">
-        <v>278</v>
+        <v>200</v>
       </c>
     </row>
     <row r="68" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B68" s="1" t="s">
-        <v>265</v>
+        <v>187</v>
       </c>
       <c r="F68" s="1" t="s">
-        <v>279</v>
+        <v>201</v>
       </c>
     </row>
     <row r="69" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B69" s="1" t="s">
-        <v>266</v>
+        <v>188</v>
       </c>
       <c r="F69" s="1" t="s">
-        <v>280</v>
+        <v>202</v>
       </c>
     </row>
     <row r="70" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B70" s="2" t="s">
-        <v>43</v>
+        <v>17</v>
       </c>
       <c r="F70" s="2" t="s">
-        <v>73</v>
+        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
sub-groups (positive - negative) visualizations added
</commit_message>
<xml_diff>
--- a/code/output/vehicle_model_results.xlsx
+++ b/code/output/vehicle_model_results.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Spring 2025\Conjoint_Survey_25\code\output\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1506456D-8A0C-4EF5-BF55-36C862BCE8CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7BC5535-AA9C-44FA-B47F-49C1CABA2A62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="3" xr2:uid="{7CCC4083-8FE9-4953-9603-647056C47B46}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="3" xr2:uid="{7CCC4083-8FE9-4953-9603-647056C47B46}"/>
   </bookViews>
   <sheets>
     <sheet name="model car || suv" sheetId="4" r:id="rId1"/>
     <sheet name="wtp models-low || high" sheetId="1" r:id="rId2"/>
     <sheet name="conf intervals-low || high" sheetId="2" r:id="rId3"/>
-    <sheet name="models pro_averse" sheetId="7" r:id="rId4"/>
+    <sheet name="models pro_averse | charger" sheetId="7" r:id="rId4"/>
     <sheet name="models-interaction" sheetId="3" r:id="rId5"/>
     <sheet name="conf intervals - interaction" sheetId="6" r:id="rId6"/>
     <sheet name="models_log_r" sheetId="5" r:id="rId7"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="572" uniqueCount="378">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="620" uniqueCount="381">
   <si>
     <t xml:space="preserve">Model Coefficients: </t>
   </si>
@@ -1176,6 +1176,15 @@
   </si>
   <si>
     <t>model_negative_group_suv</t>
+  </si>
+  <si>
+    <t>model_charger_access_yes</t>
+  </si>
+  <si>
+    <t>model_charger_access_no</t>
+  </si>
+  <si>
+    <t>model_neighbor_ev_yes</t>
   </si>
 </sst>
 </file>
@@ -1265,7 +1274,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1306,9 +1315,6 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
@@ -1333,6 +1339,16 @@
     <xf numFmtId="4" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2197,18 +2213,18 @@
   </cols>
   <sheetData>
     <row r="2" spans="3:13" x14ac:dyDescent="0.25">
-      <c r="C2" s="14" t="s">
+      <c r="C2" s="22" t="s">
         <v>9</v>
       </c>
-      <c r="D2" s="14"/>
-      <c r="E2" s="14"/>
-      <c r="F2" s="14"/>
-      <c r="H2" s="14" t="s">
+      <c r="D2" s="22"/>
+      <c r="E2" s="22"/>
+      <c r="F2" s="22"/>
+      <c r="H2" s="22" t="s">
         <v>11</v>
       </c>
-      <c r="I2" s="14"/>
-      <c r="J2" s="14"/>
-      <c r="K2" s="14"/>
+      <c r="I2" s="22"/>
+      <c r="J2" s="22"/>
+      <c r="K2" s="22"/>
     </row>
     <row r="3" spans="3:13" x14ac:dyDescent="0.25">
       <c r="C3" s="8" t="s">
@@ -2547,18 +2563,18 @@
       <c r="M14" s="6"/>
     </row>
     <row r="18" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="C18" s="14" t="s">
+      <c r="C18" s="22" t="s">
         <v>10</v>
       </c>
-      <c r="D18" s="14"/>
-      <c r="E18" s="14"/>
-      <c r="F18" s="14"/>
-      <c r="H18" s="14" t="s">
+      <c r="D18" s="22"/>
+      <c r="E18" s="22"/>
+      <c r="F18" s="22"/>
+      <c r="H18" s="22" t="s">
         <v>12</v>
       </c>
-      <c r="I18" s="14"/>
-      <c r="J18" s="14"/>
-      <c r="K18" s="14"/>
+      <c r="I18" s="22"/>
+      <c r="J18" s="22"/>
+      <c r="K18" s="22"/>
     </row>
     <row r="19" spans="3:11" x14ac:dyDescent="0.25">
       <c r="C19" s="8" t="s">
@@ -2886,40 +2902,56 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D455D975-647C-424C-912C-DB92418F2207}">
-  <dimension ref="D4:N32"/>
+  <dimension ref="D4:Y36"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="4" max="4" width="21.28515625" customWidth="1"/>
     <col min="5" max="7" width="9.85546875" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="23.5703125" customWidth="1"/>
     <col min="12" max="14" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="21.28515625" customWidth="1"/>
+    <col min="18" max="20" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="21.42578125" customWidth="1"/>
+    <col min="23" max="25" width="9.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="4" spans="4:14" x14ac:dyDescent="0.25">
-      <c r="D4" s="14" t="s">
+    <row r="4" spans="4:25" x14ac:dyDescent="0.25">
+      <c r="D4" s="22" t="s">
         <v>374</v>
       </c>
-      <c r="E4" s="14"/>
-      <c r="F4" s="14"/>
-      <c r="G4" s="14"/>
-      <c r="K4" s="14" t="s">
+      <c r="E4" s="22"/>
+      <c r="F4" s="22"/>
+      <c r="G4" s="22"/>
+      <c r="K4" s="22" t="s">
         <v>376</v>
       </c>
-      <c r="L4" s="14"/>
-      <c r="M4" s="14"/>
-      <c r="N4" s="14"/>
-    </row>
-    <row r="5" spans="4:14" x14ac:dyDescent="0.25">
-      <c r="D5" s="15" t="s">
+      <c r="L4" s="22"/>
+      <c r="M4" s="22"/>
+      <c r="N4" s="22"/>
+      <c r="Q4" s="22" t="s">
+        <v>378</v>
+      </c>
+      <c r="R4" s="22"/>
+      <c r="S4" s="22"/>
+      <c r="T4" s="22"/>
+      <c r="V4" s="22" t="s">
+        <v>379</v>
+      </c>
+      <c r="W4" s="22"/>
+      <c r="X4" s="22"/>
+      <c r="Y4" s="22"/>
+    </row>
+    <row r="5" spans="4:25" x14ac:dyDescent="0.25">
+      <c r="D5" s="14" t="s">
         <v>356</v>
       </c>
-      <c r="E5" s="16" t="s">
+      <c r="E5" s="15" t="s">
         <v>371</v>
       </c>
-      <c r="F5" s="16" t="s">
+      <c r="F5" s="15" t="s">
         <v>372</v>
       </c>
-      <c r="G5" s="16" t="s">
+      <c r="G5" s="15" t="s">
         <v>373</v>
       </c>
       <c r="K5" s="8" t="s">
@@ -2934,308 +2966,626 @@
       <c r="N5" s="9" t="s">
         <v>373</v>
       </c>
-    </row>
-    <row r="6" spans="4:14" x14ac:dyDescent="0.25">
-      <c r="D6" s="17" t="s">
+      <c r="Q5" s="23" t="s">
+        <v>356</v>
+      </c>
+      <c r="R5" s="23" t="s">
+        <v>371</v>
+      </c>
+      <c r="S5" s="23" t="s">
+        <v>372</v>
+      </c>
+      <c r="T5" s="23" t="s">
+        <v>373</v>
+      </c>
+      <c r="V5" s="14" t="s">
+        <v>356</v>
+      </c>
+      <c r="W5" s="15" t="s">
+        <v>371</v>
+      </c>
+      <c r="X5" s="15" t="s">
+        <v>372</v>
+      </c>
+      <c r="Y5" s="15" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="6" spans="4:25" x14ac:dyDescent="0.25">
+      <c r="D6" s="16" t="s">
         <v>360</v>
       </c>
-      <c r="E6" s="18">
+      <c r="E6" s="17">
         <v>-10398.52</v>
       </c>
-      <c r="F6" s="18">
+      <c r="F6" s="17">
         <v>-15013.72</v>
       </c>
-      <c r="G6" s="18">
+      <c r="G6" s="17">
         <v>-6014.7</v>
       </c>
-      <c r="K6" s="21" t="s">
+      <c r="K6" s="20" t="s">
         <v>360</v>
       </c>
-      <c r="L6" s="22">
+      <c r="L6" s="21">
         <v>-19663.169999999998</v>
       </c>
-      <c r="M6" s="22">
+      <c r="M6" s="21">
         <v>-27588.38</v>
       </c>
-      <c r="N6" s="22">
+      <c r="N6" s="21">
         <v>-12238.31</v>
       </c>
-    </row>
-    <row r="7" spans="4:14" x14ac:dyDescent="0.25">
-      <c r="D7" s="17" t="s">
+      <c r="Q6" s="16" t="s">
+        <v>360</v>
+      </c>
+      <c r="R6" s="24">
+        <v>-19530.740000000002</v>
+      </c>
+      <c r="S6" s="24">
+        <v>-23977.16</v>
+      </c>
+      <c r="T6" s="24">
+        <v>-15425.42</v>
+      </c>
+      <c r="V6" s="16" t="s">
+        <v>360</v>
+      </c>
+      <c r="W6" s="17">
+        <v>-27368.32</v>
+      </c>
+      <c r="X6" s="17">
+        <v>-31693.439999999999</v>
+      </c>
+      <c r="Y6" s="17">
+        <v>-23326.48</v>
+      </c>
+    </row>
+    <row r="7" spans="4:25" x14ac:dyDescent="0.25">
+      <c r="D7" s="16" t="s">
         <v>361</v>
       </c>
-      <c r="E7" s="18">
+      <c r="E7" s="17">
         <v>2459.6999999999998</v>
       </c>
-      <c r="F7" s="19">
+      <c r="F7" s="18">
         <v>237.23</v>
       </c>
-      <c r="G7" s="18">
+      <c r="G7" s="17">
         <v>4792.01</v>
       </c>
-      <c r="K7" s="21" t="s">
+      <c r="K7" s="20" t="s">
         <v>361</v>
       </c>
-      <c r="L7" s="22">
+      <c r="L7" s="21">
         <v>5558.54</v>
       </c>
-      <c r="M7" s="22">
+      <c r="M7" s="21">
         <v>3135.62</v>
       </c>
-      <c r="N7" s="22">
+      <c r="N7" s="21">
         <v>8116.55</v>
       </c>
-    </row>
-    <row r="8" spans="4:14" x14ac:dyDescent="0.25">
-      <c r="D8" s="17" t="s">
+      <c r="Q7" s="16" t="s">
+        <v>361</v>
+      </c>
+      <c r="R7" s="24">
+        <v>2815.85</v>
+      </c>
+      <c r="S7" s="24">
+        <v>1209.26</v>
+      </c>
+      <c r="T7" s="24">
+        <v>4451.71</v>
+      </c>
+      <c r="V7" s="16" t="s">
+        <v>361</v>
+      </c>
+      <c r="W7" s="17">
+        <v>-4797.7299999999996</v>
+      </c>
+      <c r="X7" s="17">
+        <v>-6354.98</v>
+      </c>
+      <c r="Y7" s="17">
+        <v>-3324.79</v>
+      </c>
+    </row>
+    <row r="8" spans="4:25" x14ac:dyDescent="0.25">
+      <c r="D8" s="16" t="s">
         <v>362</v>
       </c>
-      <c r="E8" s="18">
+      <c r="E8" s="17">
         <v>5936.82</v>
       </c>
-      <c r="F8" s="18">
+      <c r="F8" s="17">
         <v>3595.79</v>
       </c>
-      <c r="G8" s="18">
+      <c r="G8" s="17">
         <v>8363.34</v>
       </c>
-      <c r="K8" s="21" t="s">
+      <c r="K8" s="20" t="s">
         <v>362</v>
       </c>
-      <c r="L8" s="22">
+      <c r="L8" s="21">
         <v>6666.07</v>
       </c>
-      <c r="M8" s="22">
+      <c r="M8" s="21">
         <v>4065.63</v>
       </c>
-      <c r="N8" s="22">
+      <c r="N8" s="21">
         <v>9435.7099999999991</v>
       </c>
-    </row>
-    <row r="9" spans="4:14" x14ac:dyDescent="0.25">
-      <c r="D9" s="17" t="s">
+      <c r="Q8" s="16" t="s">
+        <v>362</v>
+      </c>
+      <c r="R8" s="24">
+        <v>4984.26</v>
+      </c>
+      <c r="S8" s="24">
+        <v>3387.17</v>
+      </c>
+      <c r="T8" s="24">
+        <v>6595.78</v>
+      </c>
+      <c r="V8" s="16" t="s">
+        <v>362</v>
+      </c>
+      <c r="W8" s="17">
+        <v>4062.85</v>
+      </c>
+      <c r="X8" s="17">
+        <v>2520.15</v>
+      </c>
+      <c r="Y8" s="17">
+        <v>5605.68</v>
+      </c>
+    </row>
+    <row r="9" spans="4:25" x14ac:dyDescent="0.25">
+      <c r="D9" s="16" t="s">
         <v>363</v>
       </c>
-      <c r="E9" s="18">
+      <c r="E9" s="17">
         <v>-2689.1</v>
       </c>
-      <c r="F9" s="18">
+      <c r="F9" s="17">
         <v>-3481.49</v>
       </c>
-      <c r="G9" s="18">
+      <c r="G9" s="17">
         <v>-2003.36</v>
       </c>
-      <c r="K9" s="21" t="s">
+      <c r="K9" s="20" t="s">
         <v>363</v>
       </c>
-      <c r="L9" s="22">
+      <c r="L9" s="21">
         <v>-3181.46</v>
       </c>
-      <c r="M9" s="22">
+      <c r="M9" s="21">
         <v>-4087.23</v>
       </c>
-      <c r="N9" s="22">
+      <c r="N9" s="21">
         <v>-2360.4699999999998</v>
       </c>
-    </row>
-    <row r="10" spans="4:14" x14ac:dyDescent="0.25">
-      <c r="D10" s="17" t="s">
+      <c r="Q9" s="16" t="s">
+        <v>363</v>
+      </c>
+      <c r="R9" s="24">
+        <v>-2579.46</v>
+      </c>
+      <c r="S9" s="24">
+        <v>-3168.32</v>
+      </c>
+      <c r="T9" s="24">
+        <v>-2036.15</v>
+      </c>
+      <c r="V9" s="16" t="s">
+        <v>363</v>
+      </c>
+      <c r="W9" s="17">
+        <v>-3220.65</v>
+      </c>
+      <c r="X9" s="17">
+        <v>-3781.23</v>
+      </c>
+      <c r="Y9" s="17">
+        <v>-2688.46</v>
+      </c>
+    </row>
+    <row r="10" spans="4:25" x14ac:dyDescent="0.25">
+      <c r="D10" s="16" t="s">
         <v>364</v>
       </c>
-      <c r="E10" s="19">
+      <c r="E10" s="18">
         <v>-990.18</v>
       </c>
-      <c r="F10" s="18">
+      <c r="F10" s="17">
         <v>-1387.19</v>
       </c>
-      <c r="G10" s="19">
+      <c r="G10" s="18">
         <v>-623.53</v>
       </c>
-      <c r="K10" s="21" t="s">
+      <c r="K10" s="20" t="s">
         <v>364</v>
       </c>
-      <c r="L10" s="22">
+      <c r="L10" s="21">
         <v>-1730.97</v>
       </c>
-      <c r="M10" s="22">
+      <c r="M10" s="21">
         <v>-2233.73</v>
       </c>
-      <c r="N10" s="22">
+      <c r="N10" s="21">
         <v>-1278.6500000000001</v>
       </c>
-    </row>
-    <row r="11" spans="4:14" x14ac:dyDescent="0.25">
-      <c r="D11" s="17" t="s">
+      <c r="Q10" s="16" t="s">
+        <v>364</v>
+      </c>
+      <c r="R10" s="24">
+        <v>-1607.9</v>
+      </c>
+      <c r="S10" s="24">
+        <v>-1951.04</v>
+      </c>
+      <c r="T10" s="24">
+        <v>-1290.6300000000001</v>
+      </c>
+      <c r="V10" s="16" t="s">
+        <v>364</v>
+      </c>
+      <c r="W10" s="17">
+        <v>-1017.65</v>
+      </c>
+      <c r="X10" s="17">
+        <v>-1300.82</v>
+      </c>
+      <c r="Y10" s="18">
+        <v>-745.07</v>
+      </c>
+    </row>
+    <row r="11" spans="4:25" x14ac:dyDescent="0.25">
+      <c r="D11" s="16" t="s">
         <v>365</v>
       </c>
-      <c r="E11" s="18">
+      <c r="E11" s="17">
         <v>-9481.4500000000007</v>
       </c>
-      <c r="F11" s="18">
+      <c r="F11" s="17">
         <v>-12697.14</v>
       </c>
-      <c r="G11" s="18">
+      <c r="G11" s="17">
         <v>-6566.78</v>
       </c>
-      <c r="K11" s="21" t="s">
+      <c r="K11" s="20" t="s">
         <v>365</v>
       </c>
-      <c r="L11" s="22">
+      <c r="L11" s="21">
         <v>-7624.87</v>
       </c>
-      <c r="M11" s="22">
+      <c r="M11" s="21">
         <v>-10744.44</v>
       </c>
-      <c r="N11" s="22">
+      <c r="N11" s="21">
         <v>-4703.42</v>
       </c>
-    </row>
-    <row r="12" spans="4:14" x14ac:dyDescent="0.25">
-      <c r="D12" s="17" t="s">
+      <c r="Q11" s="16" t="s">
+        <v>365</v>
+      </c>
+      <c r="R11" s="24">
+        <v>-7925.35</v>
+      </c>
+      <c r="S11" s="24">
+        <v>-10111.81</v>
+      </c>
+      <c r="T11" s="24">
+        <v>-5864.59</v>
+      </c>
+      <c r="V11" s="16" t="s">
+        <v>365</v>
+      </c>
+      <c r="W11" s="17">
+        <v>-7578.81</v>
+      </c>
+      <c r="X11" s="17">
+        <v>-9572.67</v>
+      </c>
+      <c r="Y11" s="17">
+        <v>-5685.36</v>
+      </c>
+    </row>
+    <row r="12" spans="4:25" x14ac:dyDescent="0.25">
+      <c r="D12" s="16" t="s">
         <v>366</v>
       </c>
-      <c r="E12" s="18">
+      <c r="E12" s="17">
         <v>-10000</v>
       </c>
-      <c r="F12" s="18">
+      <c r="F12" s="17">
         <v>-10000</v>
       </c>
-      <c r="G12" s="18">
+      <c r="G12" s="17">
         <v>-10000</v>
       </c>
-      <c r="K12" s="21" t="s">
+      <c r="K12" s="20" t="s">
         <v>366</v>
       </c>
-      <c r="L12" s="22">
+      <c r="L12" s="21">
         <v>-10000</v>
       </c>
-      <c r="M12" s="22">
+      <c r="M12" s="21">
         <v>-10000</v>
       </c>
-      <c r="N12" s="22">
+      <c r="N12" s="21">
         <v>-10000</v>
       </c>
-    </row>
-    <row r="13" spans="4:14" x14ac:dyDescent="0.25">
-      <c r="D13" s="17" t="s">
+      <c r="Q12" s="16" t="s">
+        <v>366</v>
+      </c>
+      <c r="R12" s="24">
+        <v>-10000</v>
+      </c>
+      <c r="S12" s="24">
+        <v>-10000</v>
+      </c>
+      <c r="T12" s="24">
+        <v>-10000</v>
+      </c>
+      <c r="V12" s="16" t="s">
+        <v>366</v>
+      </c>
+      <c r="W12" s="17">
+        <v>-10000</v>
+      </c>
+      <c r="X12" s="17">
+        <v>-10000</v>
+      </c>
+      <c r="Y12" s="17">
+        <v>-10000</v>
+      </c>
+    </row>
+    <row r="13" spans="4:25" x14ac:dyDescent="0.25">
+      <c r="D13" s="16" t="s">
         <v>367</v>
       </c>
-      <c r="E13" s="18">
+      <c r="E13" s="17">
         <v>-59931.26</v>
       </c>
-      <c r="F13" s="18">
+      <c r="F13" s="17">
         <v>-67975.600000000006</v>
       </c>
-      <c r="G13" s="18">
+      <c r="G13" s="17">
         <v>-53204.22</v>
       </c>
-      <c r="K13" s="21" t="s">
+      <c r="K13" s="20" t="s">
         <v>367</v>
       </c>
-      <c r="L13" s="22">
+      <c r="L13" s="21">
         <v>-67057.27</v>
       </c>
-      <c r="M13" s="22">
+      <c r="M13" s="21">
         <v>-75177.960000000006</v>
       </c>
-      <c r="N13" s="22">
+      <c r="N13" s="21">
         <v>-59804.639999999999</v>
       </c>
-    </row>
-    <row r="14" spans="4:14" x14ac:dyDescent="0.25">
-      <c r="D14" s="17" t="s">
+      <c r="Q13" s="16" t="s">
+        <v>367</v>
+      </c>
+      <c r="R13" s="24">
+        <v>-63390.92</v>
+      </c>
+      <c r="S13" s="24">
+        <v>-69049.399999999994</v>
+      </c>
+      <c r="T13" s="24">
+        <v>-58325.96</v>
+      </c>
+      <c r="V13" s="16" t="s">
+        <v>367</v>
+      </c>
+      <c r="W13" s="17">
+        <v>-65511.6</v>
+      </c>
+      <c r="X13" s="17">
+        <v>-70857.72</v>
+      </c>
+      <c r="Y13" s="17">
+        <v>-60611.38</v>
+      </c>
+    </row>
+    <row r="14" spans="4:25" x14ac:dyDescent="0.25">
+      <c r="D14" s="16" t="s">
         <v>368</v>
       </c>
-      <c r="E14" s="18">
+      <c r="E14" s="17">
         <v>-4461.7</v>
       </c>
-      <c r="F14" s="18">
+      <c r="F14" s="17">
         <v>-7357.62</v>
       </c>
-      <c r="G14" s="18">
+      <c r="G14" s="17">
         <v>-1650.52</v>
       </c>
-      <c r="K14" s="21" t="s">
+      <c r="K14" s="20" t="s">
         <v>368</v>
       </c>
-      <c r="L14" s="22">
+      <c r="L14" s="21">
         <v>-12997.1</v>
       </c>
-      <c r="M14" s="22">
+      <c r="M14" s="21">
         <v>-18474.61</v>
       </c>
-      <c r="N14" s="22">
+      <c r="N14" s="21">
         <v>-7875.77</v>
       </c>
-    </row>
-    <row r="15" spans="4:14" x14ac:dyDescent="0.25">
-      <c r="D15" s="17" t="s">
+      <c r="Q14" s="16" t="s">
+        <v>368</v>
+      </c>
+      <c r="R14" s="24">
+        <v>-14546.49</v>
+      </c>
+      <c r="S14" s="24">
+        <v>-17752.060000000001</v>
+      </c>
+      <c r="T14" s="24">
+        <v>-11617.63</v>
+      </c>
+      <c r="V14" s="16" t="s">
+        <v>368</v>
+      </c>
+      <c r="W14" s="17">
+        <v>-23305.47</v>
+      </c>
+      <c r="X14" s="17">
+        <v>-26561.9</v>
+      </c>
+      <c r="Y14" s="17">
+        <v>-20283.32</v>
+      </c>
+    </row>
+    <row r="15" spans="4:25" x14ac:dyDescent="0.25">
+      <c r="D15" s="16" t="s">
         <v>369</v>
       </c>
-      <c r="E15" s="18">
+      <c r="E15" s="17">
         <v>1475.12</v>
       </c>
-      <c r="F15" s="18">
+      <c r="F15" s="17">
         <v>-1411.39</v>
       </c>
-      <c r="G15" s="18">
+      <c r="G15" s="17">
         <v>4280.53</v>
       </c>
-      <c r="K15" s="21" t="s">
+      <c r="K15" s="20" t="s">
         <v>369</v>
       </c>
-      <c r="L15" s="22">
+      <c r="L15" s="21">
         <v>-6331.03</v>
       </c>
-      <c r="M15" s="22">
+      <c r="M15" s="21">
         <v>-9858.7000000000007</v>
       </c>
-      <c r="N15" s="22">
+      <c r="N15" s="21">
         <v>-3073.31</v>
       </c>
-    </row>
-    <row r="16" spans="4:14" x14ac:dyDescent="0.25">
-      <c r="D16" s="17" t="s">
+      <c r="Q15" s="16" t="s">
+        <v>369</v>
+      </c>
+      <c r="R15" s="24">
+        <v>-9562.23</v>
+      </c>
+      <c r="S15" s="24">
+        <v>-11981.4</v>
+      </c>
+      <c r="T15" s="24">
+        <v>-7367.93</v>
+      </c>
+      <c r="V15" s="16" t="s">
+        <v>369</v>
+      </c>
+      <c r="W15" s="17">
+        <v>-19242.62</v>
+      </c>
+      <c r="X15" s="17">
+        <v>-21994.92</v>
+      </c>
+      <c r="Y15" s="17">
+        <v>-16692.509999999998</v>
+      </c>
+    </row>
+    <row r="16" spans="4:25" x14ac:dyDescent="0.25">
+      <c r="D16" s="16" t="s">
         <v>370</v>
       </c>
-      <c r="E16" s="18">
+      <c r="E16" s="17">
         <v>7411.93</v>
       </c>
-      <c r="F16" s="18">
+      <c r="F16" s="17">
         <v>3032.78</v>
       </c>
-      <c r="G16" s="18">
+      <c r="G16" s="17">
         <v>11922.09</v>
       </c>
-      <c r="K16" s="21" t="s">
+      <c r="K16" s="20" t="s">
         <v>370</v>
       </c>
-      <c r="L16" s="21">
+      <c r="L16" s="20">
         <v>335.04</v>
       </c>
-      <c r="M16" s="22">
+      <c r="M16" s="21">
         <v>-2757.19</v>
       </c>
-      <c r="N16" s="22">
+      <c r="N16" s="21">
         <v>3380.2</v>
       </c>
-    </row>
-    <row r="20" spans="4:14" x14ac:dyDescent="0.25">
-      <c r="D20" s="14" t="s">
+      <c r="Q16" s="16" t="s">
+        <v>370</v>
+      </c>
+      <c r="R16" s="24">
+        <v>-4577.97</v>
+      </c>
+      <c r="S16" s="24">
+        <v>-7150.41</v>
+      </c>
+      <c r="T16" s="24">
+        <v>-2075.37</v>
+      </c>
+      <c r="V16" s="16" t="s">
+        <v>370</v>
+      </c>
+      <c r="W16" s="17">
+        <v>-15179.77</v>
+      </c>
+      <c r="X16" s="17">
+        <v>-18321.11</v>
+      </c>
+      <c r="Y16" s="17">
+        <v>-12275.63</v>
+      </c>
+    </row>
+    <row r="18" spans="4:24" x14ac:dyDescent="0.25">
+      <c r="Q18" s="25"/>
+      <c r="R18" s="25"/>
+      <c r="S18" s="25"/>
+      <c r="T18" s="25"/>
+      <c r="U18" s="25"/>
+      <c r="V18" s="25"/>
+      <c r="W18" s="25"/>
+      <c r="X18" s="25"/>
+    </row>
+    <row r="19" spans="4:24" x14ac:dyDescent="0.25">
+      <c r="Q19" s="25"/>
+      <c r="R19" s="25"/>
+      <c r="S19" s="25"/>
+      <c r="T19" s="25"/>
+      <c r="U19" s="25"/>
+      <c r="V19" s="25"/>
+      <c r="W19" s="25"/>
+      <c r="X19" s="25"/>
+    </row>
+    <row r="20" spans="4:24" x14ac:dyDescent="0.25">
+      <c r="D20" s="22" t="s">
         <v>375</v>
       </c>
-      <c r="E20" s="14"/>
-      <c r="F20" s="14"/>
-      <c r="G20" s="14"/>
-      <c r="K20" s="14" t="s">
+      <c r="E20" s="22"/>
+      <c r="F20" s="22"/>
+      <c r="G20" s="22"/>
+      <c r="K20" s="22" t="s">
         <v>377</v>
       </c>
-      <c r="L20" s="14"/>
-      <c r="M20" s="14"/>
-      <c r="N20" s="14"/>
-    </row>
-    <row r="21" spans="4:14" x14ac:dyDescent="0.25">
+      <c r="L20" s="22"/>
+      <c r="M20" s="22"/>
+      <c r="N20" s="22"/>
+      <c r="Q20" s="22" t="s">
+        <v>380</v>
+      </c>
+      <c r="R20" s="22"/>
+      <c r="S20" s="22"/>
+      <c r="T20" s="22"/>
+      <c r="U20" s="25"/>
+      <c r="V20" s="25"/>
+      <c r="W20" s="25"/>
+      <c r="X20" s="25"/>
+    </row>
+    <row r="21" spans="4:24" x14ac:dyDescent="0.25">
       <c r="D21" s="8" t="s">
         <v>356</v>
       </c>
@@ -3260,119 +3610,199 @@
       <c r="N21" s="9" t="s">
         <v>373</v>
       </c>
-    </row>
-    <row r="22" spans="4:14" x14ac:dyDescent="0.25">
+      <c r="Q21" s="8" t="s">
+        <v>356</v>
+      </c>
+      <c r="R21" s="9" t="s">
+        <v>371</v>
+      </c>
+      <c r="S21" s="9" t="s">
+        <v>372</v>
+      </c>
+      <c r="T21" s="9" t="s">
+        <v>373</v>
+      </c>
+      <c r="U21" s="25"/>
+      <c r="V21" s="25"/>
+      <c r="W21" s="25"/>
+      <c r="X21" s="25"/>
+    </row>
+    <row r="22" spans="4:24" x14ac:dyDescent="0.25">
       <c r="D22" s="10" t="s">
         <v>360</v>
       </c>
-      <c r="E22" s="20">
+      <c r="E22" s="19">
         <v>-21843.040000000001</v>
       </c>
-      <c r="F22" s="20">
+      <c r="F22" s="19">
         <v>-26025.27</v>
       </c>
-      <c r="G22" s="20">
+      <c r="G22" s="19">
         <v>-18077.8</v>
       </c>
       <c r="K22" s="10" t="s">
         <v>360</v>
       </c>
-      <c r="L22" s="20">
+      <c r="L22" s="19">
         <v>-37292.04</v>
       </c>
-      <c r="M22" s="20">
+      <c r="M22" s="19">
         <v>-44691.58</v>
       </c>
-      <c r="N22" s="20">
+      <c r="N22" s="19">
         <v>-30212.42</v>
       </c>
-    </row>
-    <row r="23" spans="4:14" x14ac:dyDescent="0.25">
+      <c r="Q22" s="10" t="s">
+        <v>360</v>
+      </c>
+      <c r="R22" s="19">
+        <v>-27326.18</v>
+      </c>
+      <c r="S22" s="19">
+        <v>-31588.5</v>
+      </c>
+      <c r="T22" s="19">
+        <v>-23406.9</v>
+      </c>
+      <c r="U22" s="25"/>
+      <c r="V22" s="25"/>
+      <c r="W22" s="25"/>
+      <c r="X22" s="25"/>
+    </row>
+    <row r="23" spans="4:24" x14ac:dyDescent="0.25">
       <c r="D23" s="10" t="s">
         <v>361</v>
       </c>
-      <c r="E23" s="20">
+      <c r="E23" s="19">
         <v>-3871.75</v>
       </c>
-      <c r="F23" s="20">
+      <c r="F23" s="19">
         <v>-5465.71</v>
       </c>
-      <c r="G23" s="20">
+      <c r="G23" s="19">
         <v>-2349.6999999999998</v>
       </c>
       <c r="K23" s="10" t="s">
         <v>361</v>
       </c>
-      <c r="L23" s="20">
+      <c r="L23" s="19">
         <v>-2553.63</v>
       </c>
-      <c r="M23" s="20">
+      <c r="M23" s="19">
         <v>-4293.0200000000004</v>
       </c>
       <c r="N23" s="11">
         <v>-866.01</v>
       </c>
-    </row>
-    <row r="24" spans="4:14" x14ac:dyDescent="0.25">
+      <c r="Q23" s="10" t="s">
+        <v>361</v>
+      </c>
+      <c r="R23" s="19">
+        <v>-4782.0600000000004</v>
+      </c>
+      <c r="S23" s="19">
+        <v>-6352.47</v>
+      </c>
+      <c r="T23" s="19">
+        <v>-3296.46</v>
+      </c>
+      <c r="U23" s="25"/>
+      <c r="V23" s="25"/>
+      <c r="W23" s="25"/>
+      <c r="X23" s="25"/>
+    </row>
+    <row r="24" spans="4:24" x14ac:dyDescent="0.25">
       <c r="D24" s="10" t="s">
         <v>362</v>
       </c>
-      <c r="E24" s="20">
+      <c r="E24" s="19">
         <v>2911.47</v>
       </c>
       <c r="F24" s="11">
         <v>790.28</v>
       </c>
-      <c r="G24" s="20">
+      <c r="G24" s="19">
         <v>5033.82</v>
       </c>
       <c r="K24" s="10" t="s">
         <v>362</v>
       </c>
-      <c r="L24" s="20">
+      <c r="L24" s="19">
         <v>6879.6</v>
       </c>
-      <c r="M24" s="20">
+      <c r="M24" s="19">
         <v>4530.62</v>
       </c>
-      <c r="N24" s="20">
+      <c r="N24" s="19">
         <v>9341.39</v>
       </c>
-    </row>
-    <row r="25" spans="4:14" x14ac:dyDescent="0.25">
+      <c r="Q24" s="10" t="s">
+        <v>362</v>
+      </c>
+      <c r="R24" s="19">
+        <v>4062.5</v>
+      </c>
+      <c r="S24" s="19">
+        <v>2552.02</v>
+      </c>
+      <c r="T24" s="19">
+        <v>5600.41</v>
+      </c>
+      <c r="U24" s="25"/>
+      <c r="V24" s="25"/>
+      <c r="W24" s="25"/>
+      <c r="X24" s="25"/>
+    </row>
+    <row r="25" spans="4:24" x14ac:dyDescent="0.25">
       <c r="D25" s="10" t="s">
         <v>363</v>
       </c>
-      <c r="E25" s="20">
+      <c r="E25" s="19">
         <v>-1807.76</v>
       </c>
-      <c r="F25" s="20">
+      <c r="F25" s="19">
         <v>-2297.3000000000002</v>
       </c>
-      <c r="G25" s="20">
+      <c r="G25" s="19">
         <v>-1355.81</v>
       </c>
       <c r="K25" s="10" t="s">
         <v>363</v>
       </c>
-      <c r="L25" s="20">
+      <c r="L25" s="19">
         <v>-3495.43</v>
       </c>
-      <c r="M25" s="20">
+      <c r="M25" s="19">
         <v>-4185.75</v>
       </c>
-      <c r="N25" s="20">
+      <c r="N25" s="19">
         <v>-2852.75</v>
       </c>
-    </row>
-    <row r="26" spans="4:14" x14ac:dyDescent="0.25">
+      <c r="Q25" s="10" t="s">
+        <v>363</v>
+      </c>
+      <c r="R25" s="19">
+        <v>-3213.5</v>
+      </c>
+      <c r="S25" s="19">
+        <v>-3782.8</v>
+      </c>
+      <c r="T25" s="19">
+        <v>-2678.6</v>
+      </c>
+      <c r="U25" s="25"/>
+      <c r="V25" s="25"/>
+      <c r="W25" s="25"/>
+      <c r="X25" s="25"/>
+    </row>
+    <row r="26" spans="4:24" x14ac:dyDescent="0.25">
       <c r="D26" s="10" t="s">
         <v>364</v>
       </c>
       <c r="E26" s="11">
         <v>-748.36</v>
       </c>
-      <c r="F26" s="20">
+      <c r="F26" s="19">
         <v>-1013.94</v>
       </c>
       <c r="G26" s="11">
@@ -3381,178 +3811,333 @@
       <c r="K26" s="10" t="s">
         <v>364</v>
       </c>
-      <c r="L26" s="20">
+      <c r="L26" s="19">
         <v>-1563.79</v>
       </c>
-      <c r="M26" s="20">
+      <c r="M26" s="19">
         <v>-1934.13</v>
       </c>
-      <c r="N26" s="20">
+      <c r="N26" s="19">
         <v>-1206.94</v>
       </c>
-    </row>
-    <row r="27" spans="4:14" x14ac:dyDescent="0.25">
+      <c r="Q26" s="10" t="s">
+        <v>364</v>
+      </c>
+      <c r="R26" s="19">
+        <v>-1022.35</v>
+      </c>
+      <c r="S26" s="19">
+        <v>-1309.95</v>
+      </c>
+      <c r="T26" s="11">
+        <v>-751.18</v>
+      </c>
+      <c r="U26" s="25"/>
+      <c r="V26" s="25"/>
+      <c r="W26" s="25"/>
+      <c r="X26" s="25"/>
+    </row>
+    <row r="27" spans="4:24" x14ac:dyDescent="0.25">
       <c r="D27" s="10" t="s">
         <v>365</v>
       </c>
-      <c r="E27" s="20">
+      <c r="E27" s="19">
         <v>-7843.18</v>
       </c>
-      <c r="F27" s="20">
+      <c r="F27" s="19">
         <v>-9933.56</v>
       </c>
-      <c r="G27" s="20">
+      <c r="G27" s="19">
         <v>-5906.78</v>
       </c>
       <c r="K27" s="10" t="s">
         <v>365</v>
       </c>
-      <c r="L27" s="20">
+      <c r="L27" s="19">
         <v>-8362.82</v>
       </c>
-      <c r="M27" s="20">
+      <c r="M27" s="19">
         <v>-10744.62</v>
       </c>
-      <c r="N27" s="20">
+      <c r="N27" s="19">
         <v>-6158.73</v>
       </c>
-    </row>
-    <row r="28" spans="4:14" x14ac:dyDescent="0.25">
+      <c r="Q27" s="10" t="s">
+        <v>365</v>
+      </c>
+      <c r="R27" s="19">
+        <v>-7550.88</v>
+      </c>
+      <c r="S27" s="19">
+        <v>-9554.76</v>
+      </c>
+      <c r="T27" s="19">
+        <v>-5713.17</v>
+      </c>
+      <c r="U27" s="25"/>
+      <c r="V27" s="25"/>
+      <c r="W27" s="25"/>
+      <c r="X27" s="25"/>
+    </row>
+    <row r="28" spans="4:24" x14ac:dyDescent="0.25">
       <c r="D28" s="10" t="s">
         <v>366</v>
       </c>
-      <c r="E28" s="20">
+      <c r="E28" s="19">
         <v>-10000</v>
       </c>
-      <c r="F28" s="20">
+      <c r="F28" s="19">
         <v>-10000</v>
       </c>
-      <c r="G28" s="20">
+      <c r="G28" s="19">
         <v>-10000</v>
       </c>
       <c r="K28" s="10" t="s">
         <v>366</v>
       </c>
-      <c r="L28" s="20">
+      <c r="L28" s="19">
         <v>-10000</v>
       </c>
-      <c r="M28" s="20">
+      <c r="M28" s="19">
         <v>-10000</v>
       </c>
-      <c r="N28" s="20">
+      <c r="N28" s="19">
         <v>-10000</v>
       </c>
-    </row>
-    <row r="29" spans="4:14" x14ac:dyDescent="0.25">
+      <c r="Q28" s="10" t="s">
+        <v>366</v>
+      </c>
+      <c r="R28" s="19">
+        <v>-10000</v>
+      </c>
+      <c r="S28" s="19">
+        <v>-10000</v>
+      </c>
+      <c r="T28" s="19">
+        <v>-10000</v>
+      </c>
+      <c r="U28" s="25"/>
+      <c r="V28" s="25"/>
+      <c r="W28" s="25"/>
+      <c r="X28" s="25"/>
+    </row>
+    <row r="29" spans="4:24" x14ac:dyDescent="0.25">
       <c r="D29" s="10" t="s">
         <v>367</v>
       </c>
-      <c r="E29" s="20">
+      <c r="E29" s="19">
         <v>-52707.519999999997</v>
       </c>
-      <c r="F29" s="20">
+      <c r="F29" s="19">
         <v>-57739.01</v>
       </c>
-      <c r="G29" s="20">
+      <c r="G29" s="19">
         <v>-48325.32</v>
       </c>
       <c r="K29" s="10" t="s">
         <v>367</v>
       </c>
-      <c r="L29" s="20">
+      <c r="L29" s="19">
         <v>-70028.12</v>
       </c>
-      <c r="M29" s="20">
+      <c r="M29" s="19">
         <v>-76379.990000000005</v>
       </c>
-      <c r="N29" s="20">
+      <c r="N29" s="19">
         <v>-64268.62</v>
       </c>
-    </row>
-    <row r="30" spans="4:14" x14ac:dyDescent="0.25">
+      <c r="Q29" s="10" t="s">
+        <v>367</v>
+      </c>
+      <c r="R29" s="19">
+        <v>-65448.71</v>
+      </c>
+      <c r="S29" s="19">
+        <v>-70865.210000000006</v>
+      </c>
+      <c r="T29" s="19">
+        <v>-60559.64</v>
+      </c>
+      <c r="U29" s="25"/>
+      <c r="V29" s="25"/>
+      <c r="W29" s="25"/>
+      <c r="X29" s="25"/>
+    </row>
+    <row r="30" spans="4:24" x14ac:dyDescent="0.25">
       <c r="D30" s="10" t="s">
         <v>368</v>
       </c>
-      <c r="E30" s="20">
+      <c r="E30" s="19">
         <v>-18931.57</v>
       </c>
-      <c r="F30" s="20">
+      <c r="F30" s="19">
         <v>-21858.91</v>
       </c>
-      <c r="G30" s="20">
+      <c r="G30" s="19">
         <v>-16311.9</v>
       </c>
       <c r="K30" s="10" t="s">
         <v>368</v>
       </c>
-      <c r="L30" s="20">
+      <c r="L30" s="19">
         <v>-30412.44</v>
       </c>
-      <c r="M30" s="20">
+      <c r="M30" s="19">
         <v>-35761.49</v>
       </c>
-      <c r="N30" s="20">
+      <c r="N30" s="19">
         <v>-25444.03</v>
       </c>
-    </row>
-    <row r="31" spans="4:14" x14ac:dyDescent="0.25">
+      <c r="Q30" s="10" t="s">
+        <v>368</v>
+      </c>
+      <c r="R30" s="19">
+        <v>-23263.68</v>
+      </c>
+      <c r="S30" s="19">
+        <v>-26495.200000000001</v>
+      </c>
+      <c r="T30" s="19">
+        <v>-20375.39</v>
+      </c>
+      <c r="U30" s="25"/>
+      <c r="V30" s="25"/>
+      <c r="W30" s="25"/>
+      <c r="X30" s="25"/>
+    </row>
+    <row r="31" spans="4:24" x14ac:dyDescent="0.25">
       <c r="D31" s="10" t="s">
         <v>369</v>
       </c>
-      <c r="E31" s="20">
+      <c r="E31" s="19">
         <v>-16020.11</v>
       </c>
-      <c r="F31" s="20">
+      <c r="F31" s="19">
         <v>-19065.13</v>
       </c>
-      <c r="G31" s="20">
+      <c r="G31" s="19">
         <v>-13262.47</v>
       </c>
       <c r="K31" s="10" t="s">
         <v>369</v>
       </c>
-      <c r="L31" s="20">
+      <c r="L31" s="19">
         <v>-23532.83</v>
       </c>
-      <c r="M31" s="20">
+      <c r="M31" s="19">
         <v>-27192.51</v>
       </c>
-      <c r="N31" s="20">
+      <c r="N31" s="19">
         <v>-20213.02</v>
       </c>
-    </row>
-    <row r="32" spans="4:14" x14ac:dyDescent="0.25">
+      <c r="Q31" s="10" t="s">
+        <v>369</v>
+      </c>
+      <c r="R31" s="19">
+        <v>-19201.18</v>
+      </c>
+      <c r="S31" s="19">
+        <v>-21923.94</v>
+      </c>
+      <c r="T31" s="19">
+        <v>-16768.71</v>
+      </c>
+      <c r="U31" s="25"/>
+      <c r="V31" s="25"/>
+      <c r="W31" s="25"/>
+      <c r="X31" s="25"/>
+    </row>
+    <row r="32" spans="4:24" x14ac:dyDescent="0.25">
       <c r="D32" s="10" t="s">
         <v>370</v>
       </c>
-      <c r="E32" s="20">
+      <c r="E32" s="19">
         <v>-13108.64</v>
       </c>
-      <c r="F32" s="20">
+      <c r="F32" s="19">
         <v>-17543.400000000001</v>
       </c>
-      <c r="G32" s="20">
+      <c r="G32" s="19">
         <v>-8937.5499999999993</v>
       </c>
       <c r="K32" s="10" t="s">
         <v>370</v>
       </c>
-      <c r="L32" s="20">
+      <c r="L32" s="19">
         <v>-16653.23</v>
       </c>
-      <c r="M32" s="20">
+      <c r="M32" s="19">
         <v>-19897.689999999999</v>
       </c>
-      <c r="N32" s="20">
+      <c r="N32" s="19">
         <v>-13666.57</v>
       </c>
+      <c r="Q32" s="10" t="s">
+        <v>370</v>
+      </c>
+      <c r="R32" s="19">
+        <v>-15138.69</v>
+      </c>
+      <c r="S32" s="19">
+        <v>-18266.689999999999</v>
+      </c>
+      <c r="T32" s="19">
+        <v>-12289.12</v>
+      </c>
+      <c r="U32" s="25"/>
+      <c r="V32" s="25"/>
+      <c r="W32" s="25"/>
+      <c r="X32" s="25"/>
+    </row>
+    <row r="33" spans="17:24" x14ac:dyDescent="0.25">
+      <c r="Q33" s="25"/>
+      <c r="R33" s="25"/>
+      <c r="S33" s="25"/>
+      <c r="T33" s="25"/>
+      <c r="U33" s="25"/>
+      <c r="V33" s="25"/>
+      <c r="W33" s="25"/>
+      <c r="X33" s="25"/>
+    </row>
+    <row r="34" spans="17:24" x14ac:dyDescent="0.25">
+      <c r="Q34" s="25"/>
+      <c r="R34" s="25"/>
+      <c r="S34" s="25"/>
+      <c r="T34" s="25"/>
+      <c r="U34" s="25"/>
+      <c r="V34" s="25"/>
+      <c r="W34" s="25"/>
+      <c r="X34" s="25"/>
+    </row>
+    <row r="35" spans="17:24" x14ac:dyDescent="0.25">
+      <c r="Q35" s="25"/>
+      <c r="R35" s="25"/>
+      <c r="S35" s="25"/>
+      <c r="T35" s="25"/>
+      <c r="U35" s="25"/>
+      <c r="V35" s="25"/>
+      <c r="W35" s="25"/>
+      <c r="X35" s="25"/>
+    </row>
+    <row r="36" spans="17:24" x14ac:dyDescent="0.25">
+      <c r="Q36" s="25"/>
+      <c r="R36" s="25"/>
+      <c r="S36" s="25"/>
+      <c r="T36" s="25"/>
+      <c r="U36" s="25"/>
+      <c r="V36" s="25"/>
+      <c r="W36" s="25"/>
+      <c r="X36" s="25"/>
     </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="7">
+    <mergeCell ref="V4:Y4"/>
     <mergeCell ref="D4:G4"/>
     <mergeCell ref="D20:G20"/>
     <mergeCell ref="K4:N4"/>
     <mergeCell ref="K20:N20"/>
+    <mergeCell ref="Q4:T4"/>
+    <mergeCell ref="Q20:T20"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>